<commit_message>
Int based Dictionary instead of class
</commit_message>
<xml_diff>
--- a/Assets/Database/Database.xlsx
+++ b/Assets/Database/Database.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tqhie\Unity Projects\Where-To\Assets\Database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UnityProjects\Where-To\Assets\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E50AA9DC-DC42-4C38-B083-25CF5DA07B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D18461A-261D-424D-8ABB-070FE81E4CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2772" yWindow="2088" windowWidth="17280" windowHeight="8880" xr2:uid="{0E7384ED-7C35-4E8F-B735-540A4F72621F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0E7384ED-7C35-4E8F-B735-540A4F72621F}"/>
   </bookViews>
   <sheets>
     <sheet name="RIDE_REQUEST" sheetId="3" r:id="rId1"/>
     <sheet name="NPC_ID" sheetId="1" r:id="rId2"/>
     <sheet name="LOCATION_POOL" sheetId="5" r:id="rId3"/>
     <sheet name="DIALOGUE_POOL" sheetId="2" r:id="rId4"/>
+    <sheet name="DIAG_TITLE_POOL" sheetId="6" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="NPC_IDs">NPC_ID!$A$2:$A$1048576</definedName>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="57">
   <si>
     <t>ID</t>
   </si>
@@ -92,9 +93,6 @@
     <t>END RIDE</t>
   </si>
   <si>
-    <t>na</t>
-  </si>
-  <si>
     <t>hannah.firstmet</t>
   </si>
   <si>
@@ -104,9 +102,6 @@
     <t>jimmy.default</t>
   </si>
   <si>
-    <t>jimmy.distrust</t>
-  </si>
-  <si>
     <t>jimmy.trust</t>
   </si>
   <si>
@@ -116,72 +111,12 @@
     <t>jimmy.firstmet</t>
   </si>
   <si>
-    <t>jimmy. distrust</t>
-  </si>
-  <si>
     <t>jimmy. trust</t>
   </si>
   <si>
-    <t>hannah_firstmet_geton</t>
-  </si>
-  <si>
-    <t>hannah_firstmet_ride</t>
-  </si>
-  <si>
-    <t>hannah_firstmet_end</t>
-  </si>
-  <si>
-    <t>hannah_neutral_trans</t>
-  </si>
-  <si>
-    <t>hannah_hi_one, hannah_hi_two, hannah_hi_three</t>
-  </si>
-  <si>
-    <t>hannah_yap_one, hannah_yap_two, hannah_yap_three</t>
-  </si>
-  <si>
-    <t>hannah_bye_one, hannah_bye_two, hannah_bye_three</t>
-  </si>
-  <si>
-    <t>jimmy_firstmet_geton</t>
-  </si>
-  <si>
-    <t>jimmy_firstmet_ride</t>
-  </si>
-  <si>
-    <t>jimmy_firstmet_end</t>
-  </si>
-  <si>
-    <t>jimmy_distrust_trans</t>
-  </si>
-  <si>
-    <t>jimmy_sus_geton</t>
-  </si>
-  <si>
-    <t>jimmy_sus_ride</t>
-  </si>
-  <si>
-    <t>jimmy_sus_end</t>
-  </si>
-  <si>
-    <t>jimmy_trust_trans</t>
-  </si>
-  <si>
-    <t>jimmy_trust_geton</t>
-  </si>
-  <si>
-    <t>jimmy_trust_ride</t>
-  </si>
-  <si>
-    <t>jimmy_trust_end</t>
-  </si>
-  <si>
     <t>TAG</t>
   </si>
   <si>
-    <t>05</t>
-  </si>
-  <si>
     <t>02</t>
   </si>
   <si>
@@ -200,58 +135,70 @@
     <t>00</t>
   </si>
   <si>
-    <t>4001</t>
-  </si>
-  <si>
-    <t>4002</t>
-  </si>
-  <si>
-    <t>4003</t>
-  </si>
-  <si>
-    <t>4004</t>
-  </si>
-  <si>
-    <t>4005</t>
-  </si>
-  <si>
-    <t>1001</t>
-  </si>
-  <si>
-    <t>1002</t>
-  </si>
-  <si>
-    <t>3001</t>
-  </si>
-  <si>
-    <t>3002</t>
-  </si>
-  <si>
-    <t>3003</t>
-  </si>
-  <si>
-    <t>3004</t>
-  </si>
-  <si>
-    <t>3005</t>
-  </si>
-  <si>
-    <t>2002</t>
-  </si>
-  <si>
-    <t>2003</t>
-  </si>
-  <si>
-    <t>2001</t>
-  </si>
-  <si>
-    <t>2006</t>
-  </si>
-  <si>
-    <t>2005</t>
-  </si>
-  <si>
-    <t>2004</t>
+    <t>002</t>
+  </si>
+  <si>
+    <t>001</t>
+  </si>
+  <si>
+    <t>005</t>
+  </si>
+  <si>
+    <t>003</t>
+  </si>
+  <si>
+    <t>004</t>
+  </si>
+  <si>
+    <t>006</t>
+  </si>
+  <si>
+    <t>001.transition</t>
+  </si>
+  <si>
+    <t>001.geton</t>
+  </si>
+  <si>
+    <t>001.during</t>
+  </si>
+  <si>
+    <t>001.end</t>
+  </si>
+  <si>
+    <t>002.transition</t>
+  </si>
+  <si>
+    <t>003.transition</t>
+  </si>
+  <si>
+    <t>004.transition</t>
+  </si>
+  <si>
+    <t>002.geton</t>
+  </si>
+  <si>
+    <t>003.geton</t>
+  </si>
+  <si>
+    <t>004.geton</t>
+  </si>
+  <si>
+    <t>002.during</t>
+  </si>
+  <si>
+    <t>003.during</t>
+  </si>
+  <si>
+    <t>004.during</t>
+  </si>
+  <si>
+    <t>002.end</t>
+  </si>
+  <si>
+    <t>003.end</t>
+  </si>
+  <si>
+    <t>004.end</t>
   </si>
 </sst>
 </file>
@@ -1233,16 +1180,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{847982F6-4584-4784-B812-EAA01FCD0B25}">
   <dimension ref="A1:Y44"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.5546875" style="4" customWidth="1"/>
-    <col min="2" max="6" width="12.6640625" style="4" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" style="4" customWidth="1"/>
-    <col min="8" max="10" width="12.6640625" style="8" customWidth="1"/>
-    <col min="11" max="25" width="9.109375" style="9"/>
+    <col min="1" max="1" width="17.5703125" style="4" customWidth="1"/>
+    <col min="2" max="6" width="12.7109375" style="4" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" style="4" customWidth="1"/>
+    <col min="8" max="10" width="12.7109375" style="8" customWidth="1"/>
+    <col min="11" max="25" width="9.140625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="1" customFormat="1" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:25" s="1" customFormat="1" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -1265,10 +1212,10 @@
         <v>9</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="J1" s="6"/>
       <c r="K1" s="6"/>
@@ -1287,33 +1234,33 @@
       <c r="X1" s="6"/>
       <c r="Y1" s="6"/>
     </row>
-    <row r="2" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
@@ -1332,33 +1279,33 @@
       <c r="X2" s="4"/>
       <c r="Y2" s="4"/>
     </row>
-    <row r="3" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
@@ -1377,33 +1324,33 @@
       <c r="X3" s="4"/>
       <c r="Y3" s="4"/>
     </row>
-    <row r="4" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -1422,33 +1369,33 @@
       <c r="X4" s="4"/>
       <c r="Y4" s="4"/>
     </row>
-    <row r="5" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -1467,34 +1414,7 @@
       <c r="X5" s="4"/>
       <c r="Y5" s="4"/>
     </row>
-    <row r="6" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>52</v>
-      </c>
+    <row r="6" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
@@ -1512,7 +1432,7 @@
       <c r="X6" s="4"/>
       <c r="Y6" s="4"/>
     </row>
-    <row r="7" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -1539,7 +1459,7 @@
       <c r="X7" s="4"/>
       <c r="Y7" s="4"/>
     </row>
-    <row r="8" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1566,7 +1486,7 @@
       <c r="X8" s="4"/>
       <c r="Y8" s="4"/>
     </row>
-    <row r="9" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1593,7 +1513,7 @@
       <c r="X9" s="4"/>
       <c r="Y9" s="4"/>
     </row>
-    <row r="10" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1620,7 +1540,7 @@
       <c r="X10" s="4"/>
       <c r="Y10" s="4"/>
     </row>
-    <row r="11" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1647,7 +1567,7 @@
       <c r="X11" s="4"/>
       <c r="Y11" s="4"/>
     </row>
-    <row r="12" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -1674,7 +1594,7 @@
       <c r="X12" s="4"/>
       <c r="Y12" s="4"/>
     </row>
-    <row r="13" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -1701,7 +1621,7 @@
       <c r="X13" s="4"/>
       <c r="Y13" s="4"/>
     </row>
-    <row r="14" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1728,7 +1648,7 @@
       <c r="X14" s="4"/>
       <c r="Y14" s="4"/>
     </row>
-    <row r="15" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1755,7 +1675,7 @@
       <c r="X15" s="4"/>
       <c r="Y15" s="4"/>
     </row>
-    <row r="16" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -1782,7 +1702,7 @@
       <c r="X16" s="4"/>
       <c r="Y16" s="4"/>
     </row>
-    <row r="17" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1809,7 +1729,7 @@
       <c r="X17" s="4"/>
       <c r="Y17" s="4"/>
     </row>
-    <row r="18" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -1836,7 +1756,7 @@
       <c r="X18" s="4"/>
       <c r="Y18" s="4"/>
     </row>
-    <row r="19" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1863,7 +1783,7 @@
       <c r="X19" s="4"/>
       <c r="Y19" s="4"/>
     </row>
-    <row r="20" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -1890,7 +1810,7 @@
       <c r="X20" s="4"/>
       <c r="Y20" s="4"/>
     </row>
-    <row r="21" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1917,7 +1837,7 @@
       <c r="X21" s="4"/>
       <c r="Y21" s="4"/>
     </row>
-    <row r="22" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -1944,7 +1864,7 @@
       <c r="X22" s="4"/>
       <c r="Y22" s="4"/>
     </row>
-    <row r="23" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -1971,7 +1891,7 @@
       <c r="X23" s="4"/>
       <c r="Y23" s="4"/>
     </row>
-    <row r="24" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -1998,7 +1918,7 @@
       <c r="X24" s="4"/>
       <c r="Y24" s="4"/>
     </row>
-    <row r="25" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -2025,7 +1945,7 @@
       <c r="X25" s="4"/>
       <c r="Y25" s="4"/>
     </row>
-    <row r="26" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -2052,7 +1972,7 @@
       <c r="X26" s="4"/>
       <c r="Y26" s="4"/>
     </row>
-    <row r="27" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -2079,7 +1999,7 @@
       <c r="X27" s="4"/>
       <c r="Y27" s="4"/>
     </row>
-    <row r="28" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -2106,7 +2026,7 @@
       <c r="X28" s="4"/>
       <c r="Y28" s="4"/>
     </row>
-    <row r="29" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -2133,7 +2053,7 @@
       <c r="X29" s="4"/>
       <c r="Y29" s="4"/>
     </row>
-    <row r="30" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -2160,7 +2080,7 @@
       <c r="X30" s="4"/>
       <c r="Y30" s="4"/>
     </row>
-    <row r="31" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -2187,7 +2107,7 @@
       <c r="X31" s="4"/>
       <c r="Y31" s="4"/>
     </row>
-    <row r="32" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -2214,7 +2134,7 @@
       <c r="X32" s="4"/>
       <c r="Y32" s="4"/>
     </row>
-    <row r="33" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -2241,7 +2161,7 @@
       <c r="X33" s="4"/>
       <c r="Y33" s="4"/>
     </row>
-    <row r="34" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -2268,7 +2188,7 @@
       <c r="X34" s="4"/>
       <c r="Y34" s="4"/>
     </row>
-    <row r="35" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -2295,7 +2215,7 @@
       <c r="X35" s="4"/>
       <c r="Y35" s="4"/>
     </row>
-    <row r="36" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -2322,7 +2242,7 @@
       <c r="X36" s="4"/>
       <c r="Y36" s="4"/>
     </row>
-    <row r="37" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -2349,7 +2269,7 @@
       <c r="X37" s="4"/>
       <c r="Y37" s="4"/>
     </row>
-    <row r="38" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -2376,7 +2296,7 @@
       <c r="X38" s="4"/>
       <c r="Y38" s="4"/>
     </row>
-    <row r="39" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -2403,7 +2323,7 @@
       <c r="X39" s="4"/>
       <c r="Y39" s="4"/>
     </row>
-    <row r="40" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -2430,7 +2350,7 @@
       <c r="X40" s="4"/>
       <c r="Y40" s="4"/>
     </row>
-    <row r="41" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -2457,7 +2377,7 @@
       <c r="X41" s="4"/>
       <c r="Y41" s="4"/>
     </row>
-    <row r="42" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="4"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -2484,7 +2404,7 @@
       <c r="X42" s="4"/>
       <c r="Y42" s="4"/>
     </row>
-    <row r="43" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="4"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -2511,7 +2431,7 @@
       <c r="X43" s="4"/>
       <c r="Y43" s="4"/>
     </row>
-    <row r="44" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="4"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -2541,26 +2461,23 @@
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="C2:C3" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B698B908-9440-4773-9B30-11BAE7A1734C}">
   <dimension ref="A1:X37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.33203125" style="10" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" style="10" customWidth="1"/>
-    <col min="3" max="3" width="24.109375" style="10" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" style="4" customWidth="1"/>
-    <col min="5" max="16" width="9.109375" style="4"/>
-    <col min="17" max="24" width="9.109375" style="9"/>
+    <col min="1" max="1" width="24.28515625" style="10" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" style="10" customWidth="1"/>
+    <col min="3" max="3" width="24.140625" style="10" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" style="4" customWidth="1"/>
+    <col min="5" max="16" width="9.140625" style="4"/>
+    <col min="17" max="24" width="9.140625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -2568,10 +2485,10 @@
         <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -2594,18 +2511,18 @@
       <c r="W1" s="6"/>
       <c r="X1" s="6"/>
     </row>
-    <row r="2" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
@@ -2628,18 +2545,18 @@
       <c r="W2" s="4"/>
       <c r="X2" s="4"/>
     </row>
-    <row r="3" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
@@ -2662,7 +2579,7 @@
       <c r="W3" s="4"/>
       <c r="X3" s="4"/>
     </row>
-    <row r="4" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10"/>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -2688,7 +2605,7 @@
       <c r="W4" s="4"/>
       <c r="X4" s="4"/>
     </row>
-    <row r="5" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10"/>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -2714,7 +2631,7 @@
       <c r="W5" s="4"/>
       <c r="X5" s="4"/>
     </row>
-    <row r="6" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -2740,7 +2657,7 @@
       <c r="W6" s="4"/>
       <c r="X6" s="4"/>
     </row>
-    <row r="7" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -2766,7 +2683,7 @@
       <c r="W7" s="4"/>
       <c r="X7" s="4"/>
     </row>
-    <row r="8" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -2792,7 +2709,7 @@
       <c r="W8" s="4"/>
       <c r="X8" s="4"/>
     </row>
-    <row r="9" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -2818,7 +2735,7 @@
       <c r="W9" s="4"/>
       <c r="X9" s="4"/>
     </row>
-    <row r="10" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -2844,7 +2761,7 @@
       <c r="W10" s="4"/>
       <c r="X10" s="4"/>
     </row>
-    <row r="11" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -2870,7 +2787,7 @@
       <c r="W11" s="4"/>
       <c r="X11" s="4"/>
     </row>
-    <row r="12" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -2896,7 +2813,7 @@
       <c r="W12" s="4"/>
       <c r="X12" s="4"/>
     </row>
-    <row r="13" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -2922,7 +2839,7 @@
       <c r="W13" s="4"/>
       <c r="X13" s="4"/>
     </row>
-    <row r="14" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -2948,7 +2865,7 @@
       <c r="W14" s="4"/>
       <c r="X14" s="4"/>
     </row>
-    <row r="15" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -2974,7 +2891,7 @@
       <c r="W15" s="4"/>
       <c r="X15" s="4"/>
     </row>
-    <row r="16" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -3000,7 +2917,7 @@
       <c r="W16" s="4"/>
       <c r="X16" s="4"/>
     </row>
-    <row r="17" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -3026,7 +2943,7 @@
       <c r="W17" s="4"/>
       <c r="X17" s="4"/>
     </row>
-    <row r="18" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -3052,7 +2969,7 @@
       <c r="W18" s="4"/>
       <c r="X18" s="4"/>
     </row>
-    <row r="19" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="10"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
@@ -3078,7 +2995,7 @@
       <c r="W19" s="4"/>
       <c r="X19" s="4"/>
     </row>
-    <row r="20" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="10"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
@@ -3104,7 +3021,7 @@
       <c r="W20" s="4"/>
       <c r="X20" s="4"/>
     </row>
-    <row r="21" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10"/>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
@@ -3130,7 +3047,7 @@
       <c r="W21" s="4"/>
       <c r="X21" s="4"/>
     </row>
-    <row r="22" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -3156,7 +3073,7 @@
       <c r="W22" s="4"/>
       <c r="X22" s="4"/>
     </row>
-    <row r="23" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="10"/>
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
@@ -3182,7 +3099,7 @@
       <c r="W23" s="4"/>
       <c r="X23" s="4"/>
     </row>
-    <row r="24" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="10"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
@@ -3208,7 +3125,7 @@
       <c r="W24" s="4"/>
       <c r="X24" s="4"/>
     </row>
-    <row r="25" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="10"/>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
@@ -3234,7 +3151,7 @@
       <c r="W25" s="4"/>
       <c r="X25" s="4"/>
     </row>
-    <row r="26" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="10"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
@@ -3260,7 +3177,7 @@
       <c r="W26" s="4"/>
       <c r="X26" s="4"/>
     </row>
-    <row r="27" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="10"/>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
@@ -3286,7 +3203,7 @@
       <c r="W27" s="4"/>
       <c r="X27" s="4"/>
     </row>
-    <row r="28" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
@@ -3312,7 +3229,7 @@
       <c r="W28" s="4"/>
       <c r="X28" s="4"/>
     </row>
-    <row r="29" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
@@ -3338,7 +3255,7 @@
       <c r="W29" s="4"/>
       <c r="X29" s="4"/>
     </row>
-    <row r="30" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
@@ -3364,7 +3281,7 @@
       <c r="W30" s="4"/>
       <c r="X30" s="4"/>
     </row>
-    <row r="31" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
@@ -3390,7 +3307,7 @@
       <c r="W31" s="4"/>
       <c r="X31" s="4"/>
     </row>
-    <row r="32" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="10"/>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
@@ -3416,7 +3333,7 @@
       <c r="W32" s="4"/>
       <c r="X32" s="4"/>
     </row>
-    <row r="33" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="10"/>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
@@ -3442,7 +3359,7 @@
       <c r="W33" s="4"/>
       <c r="X33" s="4"/>
     </row>
-    <row r="34" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="10"/>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
@@ -3468,7 +3385,7 @@
       <c r="W34" s="4"/>
       <c r="X34" s="4"/>
     </row>
-    <row r="35" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="10"/>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
@@ -3494,7 +3411,7 @@
       <c r="W35" s="4"/>
       <c r="X35" s="4"/>
     </row>
-    <row r="36" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="10"/>
       <c r="B36" s="10"/>
       <c r="C36" s="10"/>
@@ -3520,7 +3437,7 @@
       <c r="W36" s="4"/>
       <c r="X36" s="4"/>
     </row>
-    <row r="37" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="10"/>
       <c r="B37" s="10"/>
       <c r="C37" s="10"/>
@@ -3559,14 +3476,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EE75206-B358-44F7-8367-AB97E19840D2}">
   <dimension ref="A1:AA7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="17.33203125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" style="9" customWidth="1"/>
-    <col min="4" max="27" width="9.109375" style="9"/>
+    <col min="1" max="2" width="17.28515625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" style="9" customWidth="1"/>
+    <col min="4" max="27" width="9.140625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -3575,52 +3492,52 @@
       </c>
       <c r="C1" s="7"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>72</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -3632,15 +3549,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58DC2138-BE78-4B88-B9BC-64CC9944BEED}">
   <dimension ref="A1:O27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="22.44140625" style="15" customWidth="1"/>
-    <col min="3" max="5" width="33.5546875" style="15" customWidth="1"/>
-    <col min="6" max="6" width="33.5546875" style="16" customWidth="1"/>
-    <col min="7" max="15" width="9.109375" style="9"/>
+    <col min="1" max="2" width="22.42578125" style="15" customWidth="1"/>
+    <col min="3" max="5" width="33.5703125" style="15" customWidth="1"/>
+    <col min="6" max="6" width="33.5703125" style="16" customWidth="1"/>
+    <col min="7" max="15" width="9.140625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="3" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" s="3" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>2</v>
       </c>
@@ -3669,24 +3586,24 @@
       <c r="N1" s="14"/>
       <c r="O1" s="14"/>
     </row>
-    <row r="2" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -3698,24 +3615,24 @@
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
     </row>
-    <row r="3" spans="1:15" s="2" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -3727,24 +3644,24 @@
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
     </row>
-    <row r="4" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -3756,24 +3673,24 @@
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
     </row>
-    <row r="5" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -3785,25 +3702,13 @@
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
     </row>
-    <row r="6" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="F6" s="16" t="s">
-        <v>48</v>
-      </c>
+    <row r="6" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="15"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="16"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
@@ -3814,7 +3719,7 @@
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
     </row>
-    <row r="7" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
@@ -3831,7 +3736,7 @@
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
     </row>
-    <row r="8" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -3848,7 +3753,7 @@
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
     </row>
-    <row r="9" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="15"/>
       <c r="B9" s="15"/>
       <c r="C9" s="15"/>
@@ -3865,7 +3770,7 @@
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
     </row>
-    <row r="10" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15"/>
       <c r="B10" s="15"/>
       <c r="C10" s="15"/>
@@ -3882,7 +3787,7 @@
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
     </row>
-    <row r="11" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15"/>
       <c r="B11" s="15"/>
       <c r="C11" s="15"/>
@@ -3899,7 +3804,7 @@
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
     </row>
-    <row r="12" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="15"/>
       <c r="B12" s="15"/>
       <c r="C12" s="15"/>
@@ -3916,7 +3821,7 @@
       <c r="N12" s="4"/>
       <c r="O12" s="4"/>
     </row>
-    <row r="13" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="15"/>
       <c r="B13" s="15"/>
       <c r="C13" s="15"/>
@@ -3933,7 +3838,7 @@
       <c r="N13" s="4"/>
       <c r="O13" s="4"/>
     </row>
-    <row r="14" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="15"/>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
@@ -3950,7 +3855,7 @@
       <c r="N14" s="4"/>
       <c r="O14" s="4"/>
     </row>
-    <row r="15" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15"/>
       <c r="B15" s="15"/>
       <c r="C15" s="15"/>
@@ -3967,7 +3872,7 @@
       <c r="N15" s="4"/>
       <c r="O15" s="4"/>
     </row>
-    <row r="16" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="15"/>
       <c r="B16" s="15"/>
       <c r="C16" s="15"/>
@@ -3984,7 +3889,7 @@
       <c r="N16" s="4"/>
       <c r="O16" s="4"/>
     </row>
-    <row r="17" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="15"/>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
@@ -4001,7 +3906,7 @@
       <c r="N17" s="4"/>
       <c r="O17" s="4"/>
     </row>
-    <row r="18" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="15"/>
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
@@ -4018,7 +3923,7 @@
       <c r="N18" s="4"/>
       <c r="O18" s="4"/>
     </row>
-    <row r="19" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="15"/>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
@@ -4035,7 +3940,7 @@
       <c r="N19" s="4"/>
       <c r="O19" s="4"/>
     </row>
-    <row r="20" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="15"/>
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
@@ -4052,7 +3957,7 @@
       <c r="N20" s="4"/>
       <c r="O20" s="4"/>
     </row>
-    <row r="21" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="15"/>
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
@@ -4069,7 +3974,7 @@
       <c r="N21" s="4"/>
       <c r="O21" s="4"/>
     </row>
-    <row r="22" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="15"/>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
@@ -4086,7 +3991,7 @@
       <c r="N22" s="4"/>
       <c r="O22" s="4"/>
     </row>
-    <row r="23" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="15"/>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
@@ -4103,7 +4008,7 @@
       <c r="N23" s="4"/>
       <c r="O23" s="4"/>
     </row>
-    <row r="24" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="15"/>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
@@ -4120,7 +4025,7 @@
       <c r="N24" s="4"/>
       <c r="O24" s="4"/>
     </row>
-    <row r="25" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="15"/>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
@@ -4137,7 +4042,7 @@
       <c r="N25" s="4"/>
       <c r="O25" s="4"/>
     </row>
-    <row r="26" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="15"/>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
@@ -4154,7 +4059,7 @@
       <c r="N26" s="4"/>
       <c r="O26" s="4"/>
     </row>
-    <row r="27" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="15"/>
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
@@ -4172,7 +4077,17 @@
       <c r="O27" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F566A316-34B4-4B5B-8946-6108E462BA0B}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Request editor creation setup
</commit_message>
<xml_diff>
--- a/Assets/Database/Database.xlsx
+++ b/Assets/Database/Database.xlsx
@@ -1,34 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tqhie\Unity Projects\Where-To\Assets\Database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UnityProjects\Where-To\Assets\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C75BC0F-78C4-4FA3-9F4C-6CEFC787FD76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA4E3BF-853D-4722-932D-1A0A75E25C8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{0E7384ED-7C35-4E8F-B735-540A4F72621F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="3" xr2:uid="{0E7384ED-7C35-4E8F-B735-540A4F72621F}"/>
   </bookViews>
   <sheets>
     <sheet name="RIDE_REQUEST" sheetId="3" r:id="rId1"/>
-    <sheet name="NPC_ID" sheetId="1" r:id="rId2"/>
-    <sheet name="LOCATION_POOL" sheetId="5" r:id="rId3"/>
-    <sheet name="DIALOGUE_POOL" sheetId="2" r:id="rId4"/>
+    <sheet name="CONDITION_ID" sheetId="7" r:id="rId2"/>
+    <sheet name="DIALOGUE_POOL" sheetId="2" r:id="rId3"/>
+    <sheet name="TAGS" sheetId="8" r:id="rId4"/>
     <sheet name="DIAG_TITLE_POOL" sheetId="6" r:id="rId5"/>
+    <sheet name="NPC_ID" sheetId="1" r:id="rId6"/>
+    <sheet name="LOCATION_ID" sheetId="5" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="NPC_IDs">NPC_ID!$A$2:$A$1048576</definedName>
-    <definedName name="sadf" localSheetId="1">NPC_ID!$A$2:$A$1048576</definedName>
+    <definedName name="sadf" localSheetId="5">NPC_ID!$A$2:$A$1048576</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="92">
   <si>
     <t>ID</t>
   </si>
@@ -114,9 +116,6 @@
     <t>jimmy. trust</t>
   </si>
   <si>
-    <t>TAG</t>
-  </si>
-  <si>
     <t>02</t>
   </si>
   <si>
@@ -199,13 +198,121 @@
   </si>
   <si>
     <t>004.end</t>
+  </si>
+  <si>
+    <t>CONDITION</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>04</t>
+  </si>
+  <si>
+    <t>HANNAH_MET</t>
+  </si>
+  <si>
+    <t>INCLUDE</t>
+  </si>
+  <si>
+    <t>EXCLUDE</t>
+  </si>
+  <si>
+    <t>JIMMY_TRUSTS</t>
+  </si>
+  <si>
+    <t>DELIVERED_MESSAGE</t>
+  </si>
+  <si>
+    <t>SEGMENT</t>
+  </si>
+  <si>
+    <t>HANNAH_MET|HANNAH_ALIVE</t>
+  </si>
+  <si>
+    <t>HANNAH_DISTRUSTS|HANNAH_DEAD</t>
+  </si>
+  <si>
+    <t>JIMMY_DISTRUSTS|JIMMY_DEAD</t>
+  </si>
+  <si>
+    <t>DELIVERED_MESSAGE|JIMMY_TRUSTS</t>
+  </si>
+  <si>
+    <t>HANNAH_ALIVE</t>
+  </si>
+  <si>
+    <t>HANNAH</t>
+  </si>
+  <si>
+    <t>JIMMY</t>
+  </si>
+  <si>
+    <t>HANNAH NEUTRAL</t>
+  </si>
+  <si>
+    <t>HANNAH STRANGER</t>
+  </si>
+  <si>
+    <t>JIMMY NEUTRAL</t>
+  </si>
+  <si>
+    <t>JIMMY TRUSTS</t>
+  </si>
+  <si>
+    <t>transition_001</t>
+  </si>
+  <si>
+    <t>geton_001</t>
+  </si>
+  <si>
+    <t>during_001</t>
+  </si>
+  <si>
+    <t>end_001</t>
+  </si>
+  <si>
+    <t>transition_002</t>
+  </si>
+  <si>
+    <t>geton_002</t>
+  </si>
+  <si>
+    <t>during_002</t>
+  </si>
+  <si>
+    <t>end_002</t>
+  </si>
+  <si>
+    <t>transition_003</t>
+  </si>
+  <si>
+    <t>geton_003</t>
+  </si>
+  <si>
+    <t>during_003</t>
+  </si>
+  <si>
+    <t>end_003</t>
+  </si>
+  <si>
+    <t>end_004</t>
+  </si>
+  <si>
+    <t>during_004</t>
+  </si>
+  <si>
+    <t>geton_004</t>
+  </si>
+  <si>
+    <t>transition_004</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -359,8 +466,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -538,6 +653,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -758,7 +879,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -804,6 +925,32 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1180,16 +1327,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{847982F6-4584-4784-B812-EAA01FCD0B25}">
   <dimension ref="A1:Y44"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.5546875" style="4" customWidth="1"/>
-    <col min="2" max="6" width="12.6640625" style="4" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" style="4" customWidth="1"/>
-    <col min="8" max="10" width="12.6640625" style="8" customWidth="1"/>
-    <col min="11" max="25" width="9.109375" style="9"/>
+    <col min="1" max="1" width="17.5703125" style="4" customWidth="1"/>
+    <col min="2" max="6" width="12.7109375" style="4" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" style="8" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" style="8" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="8" customWidth="1"/>
+    <col min="11" max="25" width="9.140625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="1" customFormat="1" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:25" s="1" customFormat="1" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -1212,12 +1361,14 @@
         <v>9</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="J1" s="6"/>
+        <v>64</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>56</v>
+      </c>
       <c r="K1" s="6"/>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
@@ -1234,35 +1385,37 @@
       <c r="X1" s="6"/>
       <c r="Y1" s="6"/>
     </row>
-    <row r="2" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="D2" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F2" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>35</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>36</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>29</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J2" s="4"/>
+        <v>29</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>33</v>
+      </c>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
       <c r="M2" s="4"/>
@@ -1279,35 +1432,37 @@
       <c r="X2" s="4"/>
       <c r="Y2" s="4"/>
     </row>
-    <row r="3" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>22</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>36</v>
-      </c>
       <c r="E3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>36</v>
-      </c>
       <c r="H3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
@@ -1324,35 +1479,37 @@
       <c r="X3" s="4"/>
       <c r="Y3" s="4"/>
     </row>
-    <row r="4" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>23</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>38</v>
-      </c>
       <c r="F4" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J4" s="4"/>
+        <v>57</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>33</v>
+      </c>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
@@ -1369,35 +1526,37 @@
       <c r="X4" s="4"/>
       <c r="Y4" s="4"/>
     </row>
-    <row r="5" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>24</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>38</v>
-      </c>
       <c r="G5" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J5" s="4"/>
+        <v>58</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
@@ -1414,7 +1573,8 @@
       <c r="X5" s="4"/>
       <c r="Y5" s="4"/>
     </row>
-    <row r="6" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
@@ -1432,7 +1592,7 @@
       <c r="X6" s="4"/>
       <c r="Y6" s="4"/>
     </row>
-    <row r="7" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -1459,7 +1619,7 @@
       <c r="X7" s="4"/>
       <c r="Y7" s="4"/>
     </row>
-    <row r="8" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1486,7 +1646,7 @@
       <c r="X8" s="4"/>
       <c r="Y8" s="4"/>
     </row>
-    <row r="9" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1513,7 +1673,7 @@
       <c r="X9" s="4"/>
       <c r="Y9" s="4"/>
     </row>
-    <row r="10" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1540,7 +1700,7 @@
       <c r="X10" s="4"/>
       <c r="Y10" s="4"/>
     </row>
-    <row r="11" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1567,7 +1727,7 @@
       <c r="X11" s="4"/>
       <c r="Y11" s="4"/>
     </row>
-    <row r="12" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -1594,7 +1754,7 @@
       <c r="X12" s="4"/>
       <c r="Y12" s="4"/>
     </row>
-    <row r="13" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -1621,7 +1781,7 @@
       <c r="X13" s="4"/>
       <c r="Y13" s="4"/>
     </row>
-    <row r="14" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1648,7 +1808,7 @@
       <c r="X14" s="4"/>
       <c r="Y14" s="4"/>
     </row>
-    <row r="15" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1675,7 +1835,7 @@
       <c r="X15" s="4"/>
       <c r="Y15" s="4"/>
     </row>
-    <row r="16" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -1702,7 +1862,7 @@
       <c r="X16" s="4"/>
       <c r="Y16" s="4"/>
     </row>
-    <row r="17" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1729,7 +1889,7 @@
       <c r="X17" s="4"/>
       <c r="Y17" s="4"/>
     </row>
-    <row r="18" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -1756,7 +1916,7 @@
       <c r="X18" s="4"/>
       <c r="Y18" s="4"/>
     </row>
-    <row r="19" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1783,7 +1943,7 @@
       <c r="X19" s="4"/>
       <c r="Y19" s="4"/>
     </row>
-    <row r="20" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -1810,7 +1970,7 @@
       <c r="X20" s="4"/>
       <c r="Y20" s="4"/>
     </row>
-    <row r="21" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1837,7 +1997,7 @@
       <c r="X21" s="4"/>
       <c r="Y21" s="4"/>
     </row>
-    <row r="22" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -1864,7 +2024,7 @@
       <c r="X22" s="4"/>
       <c r="Y22" s="4"/>
     </row>
-    <row r="23" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -1891,7 +2051,7 @@
       <c r="X23" s="4"/>
       <c r="Y23" s="4"/>
     </row>
-    <row r="24" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -1918,7 +2078,7 @@
       <c r="X24" s="4"/>
       <c r="Y24" s="4"/>
     </row>
-    <row r="25" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -1945,7 +2105,7 @@
       <c r="X25" s="4"/>
       <c r="Y25" s="4"/>
     </row>
-    <row r="26" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -1972,7 +2132,7 @@
       <c r="X26" s="4"/>
       <c r="Y26" s="4"/>
     </row>
-    <row r="27" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -1999,7 +2159,7 @@
       <c r="X27" s="4"/>
       <c r="Y27" s="4"/>
     </row>
-    <row r="28" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -2026,7 +2186,7 @@
       <c r="X28" s="4"/>
       <c r="Y28" s="4"/>
     </row>
-    <row r="29" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -2053,7 +2213,7 @@
       <c r="X29" s="4"/>
       <c r="Y29" s="4"/>
     </row>
-    <row r="30" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -2080,7 +2240,7 @@
       <c r="X30" s="4"/>
       <c r="Y30" s="4"/>
     </row>
-    <row r="31" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -2107,7 +2267,7 @@
       <c r="X31" s="4"/>
       <c r="Y31" s="4"/>
     </row>
-    <row r="32" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -2134,7 +2294,7 @@
       <c r="X32" s="4"/>
       <c r="Y32" s="4"/>
     </row>
-    <row r="33" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -2161,7 +2321,7 @@
       <c r="X33" s="4"/>
       <c r="Y33" s="4"/>
     </row>
-    <row r="34" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -2188,7 +2348,7 @@
       <c r="X34" s="4"/>
       <c r="Y34" s="4"/>
     </row>
-    <row r="35" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -2215,7 +2375,7 @@
       <c r="X35" s="4"/>
       <c r="Y35" s="4"/>
     </row>
-    <row r="36" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -2242,7 +2402,7 @@
       <c r="X36" s="4"/>
       <c r="Y36" s="4"/>
     </row>
-    <row r="37" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -2269,7 +2429,7 @@
       <c r="X37" s="4"/>
       <c r="Y37" s="4"/>
     </row>
-    <row r="38" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -2296,7 +2456,7 @@
       <c r="X38" s="4"/>
       <c r="Y38" s="4"/>
     </row>
-    <row r="39" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -2323,7 +2483,7 @@
       <c r="X39" s="4"/>
       <c r="Y39" s="4"/>
     </row>
-    <row r="40" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -2350,7 +2510,7 @@
       <c r="X40" s="4"/>
       <c r="Y40" s="4"/>
     </row>
-    <row r="41" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -2377,7 +2537,7 @@
       <c r="X41" s="4"/>
       <c r="Y41" s="4"/>
     </row>
-    <row r="42" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="4"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -2404,7 +2564,7 @@
       <c r="X42" s="4"/>
       <c r="Y42" s="4"/>
     </row>
-    <row r="43" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="4"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -2431,7 +2591,7 @@
       <c r="X43" s="4"/>
       <c r="Y43" s="4"/>
     </row>
-    <row r="44" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="4"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -2465,19 +2625,918 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{961EEBF0-AFE1-4EA5-B182-201F15B5B3DF}">
+  <dimension ref="A1:C37"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.42578125" style="17" customWidth="1"/>
+    <col min="2" max="3" width="39.85546875" style="17" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="20" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+    </row>
+    <row r="5" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+    </row>
+    <row r="7" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+    </row>
+    <row r="8" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+    </row>
+    <row r="9" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+    </row>
+    <row r="10" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+    </row>
+    <row r="11" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+    </row>
+    <row r="12" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+    </row>
+    <row r="13" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+    </row>
+    <row r="14" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+    </row>
+    <row r="15" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+    </row>
+    <row r="16" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+    </row>
+    <row r="17" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+    </row>
+    <row r="18" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+    </row>
+    <row r="19" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+    </row>
+    <row r="20" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+    </row>
+    <row r="21" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+    </row>
+    <row r="22" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+    </row>
+    <row r="23" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+    </row>
+    <row r="24" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+    </row>
+    <row r="25" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+    </row>
+    <row r="26" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+    </row>
+    <row r="27" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+    </row>
+    <row r="28" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+    </row>
+    <row r="29" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+    </row>
+    <row r="30" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+    </row>
+    <row r="31" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+    </row>
+    <row r="32" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="4"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+    </row>
+    <row r="33" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+    </row>
+    <row r="34" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+    </row>
+    <row r="35" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+    </row>
+    <row r="36" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+    </row>
+    <row r="37" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="4"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58DC2138-BE78-4B88-B9BC-64CC9944BEED}">
+  <dimension ref="A1:O27"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="22.42578125" style="15" customWidth="1"/>
+    <col min="3" max="5" width="33.5703125" style="15" customWidth="1"/>
+    <col min="6" max="6" width="33.5703125" style="16" customWidth="1"/>
+    <col min="7" max="15" width="9.140625" style="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" s="3" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+    </row>
+    <row r="2" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+    </row>
+    <row r="3" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+    </row>
+    <row r="4" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+    </row>
+    <row r="5" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+    </row>
+    <row r="6" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="15"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+    </row>
+    <row r="7" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+    </row>
+    <row r="8" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+    </row>
+    <row r="9" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="15"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+    </row>
+    <row r="10" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+    </row>
+    <row r="11" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="15"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+    </row>
+    <row r="12" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="15"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+    </row>
+    <row r="13" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="15"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+    </row>
+    <row r="14" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="15"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
+    </row>
+    <row r="15" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="15"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+    </row>
+    <row r="16" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="15"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
+    </row>
+    <row r="17" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="4"/>
+    </row>
+    <row r="18" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="15"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="4"/>
+    </row>
+    <row r="19" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+    </row>
+    <row r="20" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+    </row>
+    <row r="21" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="15"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+    </row>
+    <row r="22" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="15"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
+    </row>
+    <row r="23" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="15"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4"/>
+    </row>
+    <row r="24" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="15"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+    </row>
+    <row r="25" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="15"/>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+    </row>
+    <row r="26" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="15"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="L26" s="4"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4"/>
+      <c r="O26" s="4"/>
+    </row>
+    <row r="27" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="15"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="16"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+      <c r="O27" s="4"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="20" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A799A59-169F-451F-A311-44CABBACA8B2}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" style="22" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="27"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="24"/>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="24"/>
+      <c r="B5" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="23"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F566A316-34B4-4B5B-8946-6108E462BA0B}">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.7109375" style="22" customWidth="1"/>
+    <col min="2" max="4" width="17.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="30"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B698B908-9440-4773-9B30-11BAE7A1734C}">
   <dimension ref="A1:X37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.33203125" style="10" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" style="10" customWidth="1"/>
-    <col min="3" max="3" width="24.109375" style="10" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" style="4" customWidth="1"/>
-    <col min="5" max="16" width="9.109375" style="4"/>
-    <col min="17" max="24" width="9.109375" style="9"/>
+    <col min="1" max="1" width="24.28515625" style="10" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" style="10" customWidth="1"/>
+    <col min="3" max="3" width="24.140625" style="10" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="4" customWidth="1"/>
+    <col min="6" max="16" width="9.140625" style="4"/>
+    <col min="17" max="24" width="9.140625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -2485,10 +3544,10 @@
         <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>32</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>33</v>
       </c>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -2511,18 +3570,18 @@
       <c r="W1" s="6"/>
       <c r="X1" s="6"/>
     </row>
-    <row r="2" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
@@ -2545,18 +3604,18 @@
       <c r="W2" s="4"/>
       <c r="X2" s="4"/>
     </row>
-    <row r="3" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
@@ -2579,7 +3638,7 @@
       <c r="W3" s="4"/>
       <c r="X3" s="4"/>
     </row>
-    <row r="4" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10"/>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -2605,7 +3664,7 @@
       <c r="W4" s="4"/>
       <c r="X4" s="4"/>
     </row>
-    <row r="5" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10"/>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -2631,7 +3690,7 @@
       <c r="W5" s="4"/>
       <c r="X5" s="4"/>
     </row>
-    <row r="6" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -2657,7 +3716,7 @@
       <c r="W6" s="4"/>
       <c r="X6" s="4"/>
     </row>
-    <row r="7" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -2683,7 +3742,7 @@
       <c r="W7" s="4"/>
       <c r="X7" s="4"/>
     </row>
-    <row r="8" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -2709,7 +3768,7 @@
       <c r="W8" s="4"/>
       <c r="X8" s="4"/>
     </row>
-    <row r="9" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -2735,7 +3794,7 @@
       <c r="W9" s="4"/>
       <c r="X9" s="4"/>
     </row>
-    <row r="10" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -2761,7 +3820,7 @@
       <c r="W10" s="4"/>
       <c r="X10" s="4"/>
     </row>
-    <row r="11" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -2787,7 +3846,7 @@
       <c r="W11" s="4"/>
       <c r="X11" s="4"/>
     </row>
-    <row r="12" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -2813,7 +3872,7 @@
       <c r="W12" s="4"/>
       <c r="X12" s="4"/>
     </row>
-    <row r="13" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -2839,7 +3898,7 @@
       <c r="W13" s="4"/>
       <c r="X13" s="4"/>
     </row>
-    <row r="14" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -2865,7 +3924,7 @@
       <c r="W14" s="4"/>
       <c r="X14" s="4"/>
     </row>
-    <row r="15" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -2891,7 +3950,7 @@
       <c r="W15" s="4"/>
       <c r="X15" s="4"/>
     </row>
-    <row r="16" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -2917,7 +3976,7 @@
       <c r="W16" s="4"/>
       <c r="X16" s="4"/>
     </row>
-    <row r="17" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -2943,7 +4002,7 @@
       <c r="W17" s="4"/>
       <c r="X17" s="4"/>
     </row>
-    <row r="18" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -2969,7 +4028,7 @@
       <c r="W18" s="4"/>
       <c r="X18" s="4"/>
     </row>
-    <row r="19" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="10"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
@@ -2995,7 +4054,7 @@
       <c r="W19" s="4"/>
       <c r="X19" s="4"/>
     </row>
-    <row r="20" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="10"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
@@ -3021,7 +4080,7 @@
       <c r="W20" s="4"/>
       <c r="X20" s="4"/>
     </row>
-    <row r="21" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10"/>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
@@ -3047,7 +4106,7 @@
       <c r="W21" s="4"/>
       <c r="X21" s="4"/>
     </row>
-    <row r="22" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -3073,7 +4132,7 @@
       <c r="W22" s="4"/>
       <c r="X22" s="4"/>
     </row>
-    <row r="23" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="10"/>
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
@@ -3099,7 +4158,7 @@
       <c r="W23" s="4"/>
       <c r="X23" s="4"/>
     </row>
-    <row r="24" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="10"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
@@ -3125,7 +4184,7 @@
       <c r="W24" s="4"/>
       <c r="X24" s="4"/>
     </row>
-    <row r="25" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="10"/>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
@@ -3151,7 +4210,7 @@
       <c r="W25" s="4"/>
       <c r="X25" s="4"/>
     </row>
-    <row r="26" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="10"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
@@ -3177,7 +4236,7 @@
       <c r="W26" s="4"/>
       <c r="X26" s="4"/>
     </row>
-    <row r="27" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="10"/>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
@@ -3203,7 +4262,7 @@
       <c r="W27" s="4"/>
       <c r="X27" s="4"/>
     </row>
-    <row r="28" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
@@ -3229,7 +4288,7 @@
       <c r="W28" s="4"/>
       <c r="X28" s="4"/>
     </row>
-    <row r="29" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
@@ -3255,7 +4314,7 @@
       <c r="W29" s="4"/>
       <c r="X29" s="4"/>
     </row>
-    <row r="30" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
@@ -3281,7 +4340,7 @@
       <c r="W30" s="4"/>
       <c r="X30" s="4"/>
     </row>
-    <row r="31" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
@@ -3307,7 +4366,7 @@
       <c r="W31" s="4"/>
       <c r="X31" s="4"/>
     </row>
-    <row r="32" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="10"/>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
@@ -3333,7 +4392,7 @@
       <c r="W32" s="4"/>
       <c r="X32" s="4"/>
     </row>
-    <row r="33" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="10"/>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
@@ -3359,7 +4418,7 @@
       <c r="W33" s="4"/>
       <c r="X33" s="4"/>
     </row>
-    <row r="34" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="10"/>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
@@ -3385,7 +4444,7 @@
       <c r="W34" s="4"/>
       <c r="X34" s="4"/>
     </row>
-    <row r="35" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="10"/>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
@@ -3411,7 +4470,7 @@
       <c r="W35" s="4"/>
       <c r="X35" s="4"/>
     </row>
-    <row r="36" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="10"/>
       <c r="B36" s="10"/>
       <c r="C36" s="10"/>
@@ -3437,7 +4496,7 @@
       <c r="W36" s="4"/>
       <c r="X36" s="4"/>
     </row>
-    <row r="37" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="10"/>
       <c r="B37" s="10"/>
       <c r="C37" s="10"/>
@@ -3473,17 +4532,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EE75206-B358-44F7-8367-AB97E19840D2}">
   <dimension ref="A1:AA7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="17.33203125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" style="9" customWidth="1"/>
-    <col min="4" max="27" width="9.109375" style="9"/>
+    <col min="1" max="2" width="17.28515625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" style="9" customWidth="1"/>
+    <col min="4" max="27" width="9.140625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -3492,602 +4551,56 @@
       </c>
       <c r="C1" s="7"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58DC2138-BE78-4B88-B9BC-64CC9944BEED}">
-  <dimension ref="A1:O27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="2" width="22.44140625" style="15" customWidth="1"/>
-    <col min="3" max="5" width="33.5546875" style="15" customWidth="1"/>
-    <col min="6" max="6" width="33.5546875" style="16" customWidth="1"/>
-    <col min="7" max="15" width="9.109375" style="9"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15" s="3" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
-    </row>
-    <row r="2" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="F2" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-    </row>
-    <row r="3" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-    </row>
-    <row r="4" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
-    </row>
-    <row r="5" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-    </row>
-    <row r="6" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="15"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
-    </row>
-    <row r="7" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="15"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
-    </row>
-    <row r="8" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="15"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
-    </row>
-    <row r="9" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="15"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
-    </row>
-    <row r="10" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="15"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
-      <c r="O10" s="4"/>
-    </row>
-    <row r="11" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
-      <c r="N11" s="4"/>
-      <c r="O11" s="4"/>
-    </row>
-    <row r="12" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="15"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
-    </row>
-    <row r="13" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="15"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
-      <c r="N13" s="4"/>
-      <c r="O13" s="4"/>
-    </row>
-    <row r="14" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="15"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
-    </row>
-    <row r="15" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="15"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
-      <c r="O15" s="4"/>
-    </row>
-    <row r="16" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="15"/>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
-      <c r="N16" s="4"/>
-      <c r="O16" s="4"/>
-    </row>
-    <row r="17" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="15"/>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
-      <c r="N17" s="4"/>
-      <c r="O17" s="4"/>
-    </row>
-    <row r="18" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="15"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="4"/>
-    </row>
-    <row r="19" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="15"/>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="M19" s="4"/>
-      <c r="N19" s="4"/>
-      <c r="O19" s="4"/>
-    </row>
-    <row r="20" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="15"/>
-      <c r="B20" s="15"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
-      <c r="M20" s="4"/>
-      <c r="N20" s="4"/>
-      <c r="O20" s="4"/>
-    </row>
-    <row r="21" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="15"/>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
-      <c r="M21" s="4"/>
-      <c r="N21" s="4"/>
-      <c r="O21" s="4"/>
-    </row>
-    <row r="22" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="15"/>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
-      <c r="M22" s="4"/>
-      <c r="N22" s="4"/>
-      <c r="O22" s="4"/>
-    </row>
-    <row r="23" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="15"/>
-      <c r="B23" s="15"/>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
-      <c r="M23" s="4"/>
-      <c r="N23" s="4"/>
-      <c r="O23" s="4"/>
-    </row>
-    <row r="24" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="15"/>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
-      <c r="L24" s="4"/>
-      <c r="M24" s="4"/>
-      <c r="N24" s="4"/>
-      <c r="O24" s="4"/>
-    </row>
-    <row r="25" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="15"/>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4"/>
-      <c r="L25" s="4"/>
-      <c r="M25" s="4"/>
-      <c r="N25" s="4"/>
-      <c r="O25" s="4"/>
-    </row>
-    <row r="26" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="15"/>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
-      <c r="L26" s="4"/>
-      <c r="M26" s="4"/>
-      <c r="N26" s="4"/>
-      <c r="O26" s="4"/>
-    </row>
-    <row r="27" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="15"/>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-      <c r="L27" s="4"/>
-      <c r="M27" s="4"/>
-      <c r="N27" s="4"/>
-      <c r="O27" s="4"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="20" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F566A316-34B4-4B5B-8946-6108E462BA0B}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Ride reqest creation done, world state and selection logic in progress
</commit_message>
<xml_diff>
--- a/Assets/Database/Database.xlsx
+++ b/Assets/Database/Database.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UnityProjects\Where-To\Assets\Database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tqhie\Unity Projects\Where-To\Assets\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA4E3BF-853D-4722-932D-1A0A75E25C8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="3" xr2:uid="{0E7384ED-7C35-4E8F-B735-540A4F72621F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="2" xr2:uid="{0E7384ED-7C35-4E8F-B735-540A4F72621F}"/>
   </bookViews>
   <sheets>
     <sheet name="RIDE_REQUEST" sheetId="3" r:id="rId1"/>
@@ -879,7 +879,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -942,15 +942,11 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1327,18 +1323,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{847982F6-4584-4784-B812-EAA01FCD0B25}">
   <dimension ref="A1:Y44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" style="4" customWidth="1"/>
-    <col min="2" max="6" width="12.7109375" style="4" customWidth="1"/>
-    <col min="7" max="7" width="16.28515625" style="4" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" style="8" customWidth="1"/>
-    <col min="9" max="9" width="15.42578125" style="8" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" style="8" customWidth="1"/>
-    <col min="11" max="25" width="9.140625" style="9"/>
+    <col min="1" max="1" width="17.5546875" style="4" customWidth="1"/>
+    <col min="2" max="6" width="12.6640625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" style="4" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" style="8" customWidth="1"/>
+    <col min="9" max="9" width="15.44140625" style="8" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" style="8" customWidth="1"/>
+    <col min="11" max="25" width="9.109375" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="1" customFormat="1" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" s="1" customFormat="1" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -1385,7 +1381,7 @@
       <c r="X1" s="6"/>
       <c r="Y1" s="6"/>
     </row>
-    <row r="2" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>21</v>
       </c>
@@ -1432,7 +1428,7 @@
       <c r="X2" s="4"/>
       <c r="Y2" s="4"/>
     </row>
-    <row r="3" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>22</v>
       </c>
@@ -1479,7 +1475,7 @@
       <c r="X3" s="4"/>
       <c r="Y3" s="4"/>
     </row>
-    <row r="4" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>23</v>
       </c>
@@ -1526,7 +1522,7 @@
       <c r="X4" s="4"/>
       <c r="Y4" s="4"/>
     </row>
-    <row r="5" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>24</v>
       </c>
@@ -1573,7 +1569,7 @@
       <c r="X5" s="4"/>
       <c r="Y5" s="4"/>
     </row>
-    <row r="6" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -1592,7 +1588,7 @@
       <c r="X6" s="4"/>
       <c r="Y6" s="4"/>
     </row>
-    <row r="7" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -1619,7 +1615,7 @@
       <c r="X7" s="4"/>
       <c r="Y7" s="4"/>
     </row>
-    <row r="8" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1646,7 +1642,7 @@
       <c r="X8" s="4"/>
       <c r="Y8" s="4"/>
     </row>
-    <row r="9" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1673,7 +1669,7 @@
       <c r="X9" s="4"/>
       <c r="Y9" s="4"/>
     </row>
-    <row r="10" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1700,7 +1696,7 @@
       <c r="X10" s="4"/>
       <c r="Y10" s="4"/>
     </row>
-    <row r="11" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1727,7 +1723,7 @@
       <c r="X11" s="4"/>
       <c r="Y11" s="4"/>
     </row>
-    <row r="12" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -1754,7 +1750,7 @@
       <c r="X12" s="4"/>
       <c r="Y12" s="4"/>
     </row>
-    <row r="13" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -1781,7 +1777,7 @@
       <c r="X13" s="4"/>
       <c r="Y13" s="4"/>
     </row>
-    <row r="14" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1808,7 +1804,7 @@
       <c r="X14" s="4"/>
       <c r="Y14" s="4"/>
     </row>
-    <row r="15" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1835,7 +1831,7 @@
       <c r="X15" s="4"/>
       <c r="Y15" s="4"/>
     </row>
-    <row r="16" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -1862,7 +1858,7 @@
       <c r="X16" s="4"/>
       <c r="Y16" s="4"/>
     </row>
-    <row r="17" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1889,7 +1885,7 @@
       <c r="X17" s="4"/>
       <c r="Y17" s="4"/>
     </row>
-    <row r="18" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -1916,7 +1912,7 @@
       <c r="X18" s="4"/>
       <c r="Y18" s="4"/>
     </row>
-    <row r="19" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1943,7 +1939,7 @@
       <c r="X19" s="4"/>
       <c r="Y19" s="4"/>
     </row>
-    <row r="20" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -1970,7 +1966,7 @@
       <c r="X20" s="4"/>
       <c r="Y20" s="4"/>
     </row>
-    <row r="21" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1997,7 +1993,7 @@
       <c r="X21" s="4"/>
       <c r="Y21" s="4"/>
     </row>
-    <row r="22" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -2024,7 +2020,7 @@
       <c r="X22" s="4"/>
       <c r="Y22" s="4"/>
     </row>
-    <row r="23" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -2051,7 +2047,7 @@
       <c r="X23" s="4"/>
       <c r="Y23" s="4"/>
     </row>
-    <row r="24" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -2078,7 +2074,7 @@
       <c r="X24" s="4"/>
       <c r="Y24" s="4"/>
     </row>
-    <row r="25" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -2105,7 +2101,7 @@
       <c r="X25" s="4"/>
       <c r="Y25" s="4"/>
     </row>
-    <row r="26" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -2132,7 +2128,7 @@
       <c r="X26" s="4"/>
       <c r="Y26" s="4"/>
     </row>
-    <row r="27" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -2159,7 +2155,7 @@
       <c r="X27" s="4"/>
       <c r="Y27" s="4"/>
     </row>
-    <row r="28" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -2186,7 +2182,7 @@
       <c r="X28" s="4"/>
       <c r="Y28" s="4"/>
     </row>
-    <row r="29" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -2213,7 +2209,7 @@
       <c r="X29" s="4"/>
       <c r="Y29" s="4"/>
     </row>
-    <row r="30" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -2240,7 +2236,7 @@
       <c r="X30" s="4"/>
       <c r="Y30" s="4"/>
     </row>
-    <row r="31" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -2267,7 +2263,7 @@
       <c r="X31" s="4"/>
       <c r="Y31" s="4"/>
     </row>
-    <row r="32" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -2294,7 +2290,7 @@
       <c r="X32" s="4"/>
       <c r="Y32" s="4"/>
     </row>
-    <row r="33" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -2321,7 +2317,7 @@
       <c r="X33" s="4"/>
       <c r="Y33" s="4"/>
     </row>
-    <row r="34" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -2348,7 +2344,7 @@
       <c r="X34" s="4"/>
       <c r="Y34" s="4"/>
     </row>
-    <row r="35" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -2375,7 +2371,7 @@
       <c r="X35" s="4"/>
       <c r="Y35" s="4"/>
     </row>
-    <row r="36" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -2402,7 +2398,7 @@
       <c r="X36" s="4"/>
       <c r="Y36" s="4"/>
     </row>
-    <row r="37" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -2429,7 +2425,7 @@
       <c r="X37" s="4"/>
       <c r="Y37" s="4"/>
     </row>
-    <row r="38" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -2456,7 +2452,7 @@
       <c r="X38" s="4"/>
       <c r="Y38" s="4"/>
     </row>
-    <row r="39" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -2483,7 +2479,7 @@
       <c r="X39" s="4"/>
       <c r="Y39" s="4"/>
     </row>
-    <row r="40" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -2510,7 +2506,7 @@
       <c r="X40" s="4"/>
       <c r="Y40" s="4"/>
     </row>
-    <row r="41" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -2537,7 +2533,7 @@
       <c r="X41" s="4"/>
       <c r="Y41" s="4"/>
     </row>
-    <row r="42" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -2564,7 +2560,7 @@
       <c r="X42" s="4"/>
       <c r="Y42" s="4"/>
     </row>
-    <row r="43" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -2591,7 +2587,7 @@
       <c r="X43" s="4"/>
       <c r="Y43" s="4"/>
     </row>
-    <row r="44" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -2627,13 +2623,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{961EEBF0-AFE1-4EA5-B182-201F15B5B3DF}">
   <dimension ref="A1:C37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.42578125" style="17" customWidth="1"/>
-    <col min="2" max="3" width="39.85546875" style="17" customWidth="1"/>
+    <col min="1" max="1" width="19.44140625" style="17" customWidth="1"/>
+    <col min="2" max="3" width="39.88671875" style="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="20" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="20" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -2644,7 +2640,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>29</v>
       </c>
@@ -2655,7 +2651,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>28</v>
       </c>
@@ -2666,172 +2662,172 @@
         <v>67</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
     </row>
-    <row r="5" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
     </row>
-    <row r="6" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
     </row>
-    <row r="7" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
     </row>
-    <row r="8" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
     </row>
-    <row r="9" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
     </row>
-    <row r="10" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
     </row>
-    <row r="11" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
     </row>
-    <row r="12" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
     </row>
-    <row r="14" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
     </row>
-    <row r="15" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
     </row>
-    <row r="16" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
     </row>
-    <row r="17" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
     </row>
-    <row r="18" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
     </row>
-    <row r="19" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
     </row>
-    <row r="20" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
     </row>
-    <row r="21" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
     </row>
-    <row r="22" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
     </row>
-    <row r="23" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
     </row>
-    <row r="24" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
     </row>
-    <row r="25" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
     </row>
-    <row r="26" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
     </row>
-    <row r="27" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
     </row>
-    <row r="28" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
     </row>
-    <row r="29" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
     </row>
-    <row r="30" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
     </row>
-    <row r="31" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
     </row>
-    <row r="32" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
     </row>
-    <row r="33" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
     </row>
-    <row r="34" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
     </row>
-    <row r="35" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
     </row>
-    <row r="36" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
     </row>
-    <row r="37" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -2844,15 +2840,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58DC2138-BE78-4B88-B9BC-64CC9944BEED}">
   <dimension ref="A1:O27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="22.42578125" style="15" customWidth="1"/>
-    <col min="3" max="5" width="33.5703125" style="15" customWidth="1"/>
-    <col min="6" max="6" width="33.5703125" style="16" customWidth="1"/>
-    <col min="7" max="15" width="9.140625" style="9"/>
+    <col min="1" max="2" width="22.44140625" style="15" customWidth="1"/>
+    <col min="3" max="5" width="33.5546875" style="15" customWidth="1"/>
+    <col min="6" max="6" width="33.5546875" style="16" customWidth="1"/>
+    <col min="7" max="15" width="9.109375" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="3" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" s="3" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>2</v>
       </c>
@@ -2881,7 +2877,7 @@
       <c r="N1" s="14"/>
       <c r="O1" s="14"/>
     </row>
-    <row r="2" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
         <v>21</v>
       </c>
@@ -2910,7 +2906,7 @@
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
     </row>
-    <row r="3" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
         <v>25</v>
       </c>
@@ -2939,7 +2935,7 @@
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
     </row>
-    <row r="4" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
         <v>26</v>
       </c>
@@ -2968,7 +2964,7 @@
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
     </row>
-    <row r="5" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
         <v>27</v>
       </c>
@@ -2997,7 +2993,7 @@
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
     </row>
-    <row r="6" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="15"/>
       <c r="B6" s="15"/>
       <c r="C6" s="15"/>
@@ -3014,7 +3010,7 @@
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
     </row>
-    <row r="7" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
@@ -3031,7 +3027,7 @@
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
     </row>
-    <row r="8" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -3048,7 +3044,7 @@
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
     </row>
-    <row r="9" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="15"/>
       <c r="B9" s="15"/>
       <c r="C9" s="15"/>
@@ -3065,7 +3061,7 @@
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
     </row>
-    <row r="10" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="15"/>
       <c r="B10" s="15"/>
       <c r="C10" s="15"/>
@@ -3082,7 +3078,7 @@
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
     </row>
-    <row r="11" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="15"/>
       <c r="B11" s="15"/>
       <c r="C11" s="15"/>
@@ -3099,7 +3095,7 @@
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
     </row>
-    <row r="12" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="15"/>
       <c r="B12" s="15"/>
       <c r="C12" s="15"/>
@@ -3116,7 +3112,7 @@
       <c r="N12" s="4"/>
       <c r="O12" s="4"/>
     </row>
-    <row r="13" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="15"/>
       <c r="B13" s="15"/>
       <c r="C13" s="15"/>
@@ -3133,7 +3129,7 @@
       <c r="N13" s="4"/>
       <c r="O13" s="4"/>
     </row>
-    <row r="14" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="15"/>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
@@ -3150,7 +3146,7 @@
       <c r="N14" s="4"/>
       <c r="O14" s="4"/>
     </row>
-    <row r="15" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="15"/>
       <c r="B15" s="15"/>
       <c r="C15" s="15"/>
@@ -3167,7 +3163,7 @@
       <c r="N15" s="4"/>
       <c r="O15" s="4"/>
     </row>
-    <row r="16" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="15"/>
       <c r="B16" s="15"/>
       <c r="C16" s="15"/>
@@ -3184,7 +3180,7 @@
       <c r="N16" s="4"/>
       <c r="O16" s="4"/>
     </row>
-    <row r="17" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="15"/>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
@@ -3201,7 +3197,7 @@
       <c r="N17" s="4"/>
       <c r="O17" s="4"/>
     </row>
-    <row r="18" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="15"/>
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
@@ -3218,7 +3214,7 @@
       <c r="N18" s="4"/>
       <c r="O18" s="4"/>
     </row>
-    <row r="19" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="15"/>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
@@ -3235,7 +3231,7 @@
       <c r="N19" s="4"/>
       <c r="O19" s="4"/>
     </row>
-    <row r="20" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="15"/>
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
@@ -3252,7 +3248,7 @@
       <c r="N20" s="4"/>
       <c r="O20" s="4"/>
     </row>
-    <row r="21" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="15"/>
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
@@ -3269,7 +3265,7 @@
       <c r="N21" s="4"/>
       <c r="O21" s="4"/>
     </row>
-    <row r="22" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="15"/>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
@@ -3286,7 +3282,7 @@
       <c r="N22" s="4"/>
       <c r="O22" s="4"/>
     </row>
-    <row r="23" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="15"/>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
@@ -3303,7 +3299,7 @@
       <c r="N23" s="4"/>
       <c r="O23" s="4"/>
     </row>
-    <row r="24" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="15"/>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
@@ -3320,7 +3316,7 @@
       <c r="N24" s="4"/>
       <c r="O24" s="4"/>
     </row>
-    <row r="25" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="15"/>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
@@ -3337,7 +3333,7 @@
       <c r="N25" s="4"/>
       <c r="O25" s="4"/>
     </row>
-    <row r="26" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="15"/>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
@@ -3354,7 +3350,7 @@
       <c r="N26" s="4"/>
       <c r="O26" s="4"/>
     </row>
-    <row r="27" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="15"/>
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
@@ -3381,47 +3377,47 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A799A59-169F-451F-A311-44CABBACA8B2}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" style="22" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" customWidth="1"/>
+    <col min="1" max="1" width="15.88671875" style="22" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="29" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27"/>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="25"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="26" t="s">
         <v>70</v>
       </c>
       <c r="B2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="24"/>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="26"/>
       <c r="B3" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="24" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="26" t="s">
         <v>71</v>
       </c>
       <c r="B4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="24"/>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="26"/>
       <c r="B5" s="4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
     </row>
   </sheetData>
@@ -3436,20 +3432,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F566A316-34B4-4B5B-8946-6108E462BA0B}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="22" customWidth="1"/>
-    <col min="2" max="4" width="17.140625" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" style="22" customWidth="1"/>
+    <col min="2" max="4" width="17.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="25" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30"/>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="25"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
         <v>73</v>
       </c>
@@ -3466,7 +3462,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
         <v>72</v>
       </c>
@@ -3483,7 +3479,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
         <v>74</v>
       </c>
@@ -3500,7 +3496,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
         <v>75</v>
       </c>
@@ -3525,18 +3521,18 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B698B908-9440-4773-9B30-11BAE7A1734C}">
   <dimension ref="A1:X37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.28515625" style="10" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="10" customWidth="1"/>
-    <col min="3" max="3" width="24.140625" style="10" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="4" customWidth="1"/>
-    <col min="6" max="16" width="9.140625" style="4"/>
-    <col min="17" max="24" width="9.140625" style="9"/>
+    <col min="1" max="1" width="24.33203125" style="10" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" style="10" customWidth="1"/>
+    <col min="3" max="3" width="24.109375" style="10" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" style="4" customWidth="1"/>
+    <col min="6" max="16" width="9.109375" style="4"/>
+    <col min="17" max="24" width="9.109375" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -3570,7 +3566,7 @@
       <c r="W1" s="6"/>
       <c r="X1" s="6"/>
     </row>
-    <row r="2" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -3604,7 +3600,7 @@
       <c r="W2" s="4"/>
       <c r="X2" s="4"/>
     </row>
-    <row r="3" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>5</v>
       </c>
@@ -3638,7 +3634,7 @@
       <c r="W3" s="4"/>
       <c r="X3" s="4"/>
     </row>
-    <row r="4" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -3664,7 +3660,7 @@
       <c r="W4" s="4"/>
       <c r="X4" s="4"/>
     </row>
-    <row r="5" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10"/>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -3690,7 +3686,7 @@
       <c r="W5" s="4"/>
       <c r="X5" s="4"/>
     </row>
-    <row r="6" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -3716,7 +3712,7 @@
       <c r="W6" s="4"/>
       <c r="X6" s="4"/>
     </row>
-    <row r="7" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -3742,7 +3738,7 @@
       <c r="W7" s="4"/>
       <c r="X7" s="4"/>
     </row>
-    <row r="8" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -3768,7 +3764,7 @@
       <c r="W8" s="4"/>
       <c r="X8" s="4"/>
     </row>
-    <row r="9" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -3794,7 +3790,7 @@
       <c r="W9" s="4"/>
       <c r="X9" s="4"/>
     </row>
-    <row r="10" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -3820,7 +3816,7 @@
       <c r="W10" s="4"/>
       <c r="X10" s="4"/>
     </row>
-    <row r="11" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -3846,7 +3842,7 @@
       <c r="W11" s="4"/>
       <c r="X11" s="4"/>
     </row>
-    <row r="12" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -3872,7 +3868,7 @@
       <c r="W12" s="4"/>
       <c r="X12" s="4"/>
     </row>
-    <row r="13" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -3898,7 +3894,7 @@
       <c r="W13" s="4"/>
       <c r="X13" s="4"/>
     </row>
-    <row r="14" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -3924,7 +3920,7 @@
       <c r="W14" s="4"/>
       <c r="X14" s="4"/>
     </row>
-    <row r="15" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -3950,7 +3946,7 @@
       <c r="W15" s="4"/>
       <c r="X15" s="4"/>
     </row>
-    <row r="16" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -3976,7 +3972,7 @@
       <c r="W16" s="4"/>
       <c r="X16" s="4"/>
     </row>
-    <row r="17" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -4002,7 +3998,7 @@
       <c r="W17" s="4"/>
       <c r="X17" s="4"/>
     </row>
-    <row r="18" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -4028,7 +4024,7 @@
       <c r="W18" s="4"/>
       <c r="X18" s="4"/>
     </row>
-    <row r="19" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="10"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
@@ -4054,7 +4050,7 @@
       <c r="W19" s="4"/>
       <c r="X19" s="4"/>
     </row>
-    <row r="20" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="10"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
@@ -4080,7 +4076,7 @@
       <c r="W20" s="4"/>
       <c r="X20" s="4"/>
     </row>
-    <row r="21" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="10"/>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
@@ -4106,7 +4102,7 @@
       <c r="W21" s="4"/>
       <c r="X21" s="4"/>
     </row>
-    <row r="22" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -4132,7 +4128,7 @@
       <c r="W22" s="4"/>
       <c r="X22" s="4"/>
     </row>
-    <row r="23" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="10"/>
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
@@ -4158,7 +4154,7 @@
       <c r="W23" s="4"/>
       <c r="X23" s="4"/>
     </row>
-    <row r="24" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
@@ -4184,7 +4180,7 @@
       <c r="W24" s="4"/>
       <c r="X24" s="4"/>
     </row>
-    <row r="25" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="10"/>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
@@ -4210,7 +4206,7 @@
       <c r="W25" s="4"/>
       <c r="X25" s="4"/>
     </row>
-    <row r="26" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="10"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
@@ -4236,7 +4232,7 @@
       <c r="W26" s="4"/>
       <c r="X26" s="4"/>
     </row>
-    <row r="27" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="10"/>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
@@ -4262,7 +4258,7 @@
       <c r="W27" s="4"/>
       <c r="X27" s="4"/>
     </row>
-    <row r="28" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
@@ -4288,7 +4284,7 @@
       <c r="W28" s="4"/>
       <c r="X28" s="4"/>
     </row>
-    <row r="29" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
@@ -4314,7 +4310,7 @@
       <c r="W29" s="4"/>
       <c r="X29" s="4"/>
     </row>
-    <row r="30" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
@@ -4340,7 +4336,7 @@
       <c r="W30" s="4"/>
       <c r="X30" s="4"/>
     </row>
-    <row r="31" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
@@ -4366,7 +4362,7 @@
       <c r="W31" s="4"/>
       <c r="X31" s="4"/>
     </row>
-    <row r="32" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="10"/>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
@@ -4392,7 +4388,7 @@
       <c r="W32" s="4"/>
       <c r="X32" s="4"/>
     </row>
-    <row r="33" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
@@ -4418,7 +4414,7 @@
       <c r="W33" s="4"/>
       <c r="X33" s="4"/>
     </row>
-    <row r="34" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="10"/>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
@@ -4444,7 +4440,7 @@
       <c r="W34" s="4"/>
       <c r="X34" s="4"/>
     </row>
-    <row r="35" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="10"/>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
@@ -4470,7 +4466,7 @@
       <c r="W35" s="4"/>
       <c r="X35" s="4"/>
     </row>
-    <row r="36" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="10"/>
       <c r="B36" s="10"/>
       <c r="C36" s="10"/>
@@ -4496,7 +4492,7 @@
       <c r="W36" s="4"/>
       <c r="X36" s="4"/>
     </row>
-    <row r="37" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="10"/>
       <c r="B37" s="10"/>
       <c r="C37" s="10"/>
@@ -4535,14 +4531,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EE75206-B358-44F7-8367-AB97E19840D2}">
   <dimension ref="A1:AA7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="17.28515625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" style="9" customWidth="1"/>
-    <col min="4" max="27" width="9.140625" style="9"/>
+    <col min="1" max="2" width="17.33203125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" style="9" customWidth="1"/>
+    <col min="4" max="27" width="9.109375" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -4551,7 +4547,7 @@
       </c>
       <c r="C1" s="7"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
@@ -4559,7 +4555,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>11</v>
       </c>
@@ -4567,7 +4563,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
@@ -4575,7 +4571,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
@@ -4583,7 +4579,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>14</v>
       </c>
@@ -4591,7 +4587,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
commented out condition parsing and merge world state to old system
</commit_message>
<xml_diff>
--- a/Assets/Database/Database.xlsx
+++ b/Assets/Database/Database.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tqhie\Unity Projects\Where-To\Assets\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C75BC0F-78C4-4FA3-9F4C-6CEFC787FD76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C573A222-278D-49D9-9CC6-8ECB310BA040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{0E7384ED-7C35-4E8F-B735-540A4F72621F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0E7384ED-7C35-4E8F-B735-540A4F72621F}"/>
   </bookViews>
   <sheets>
     <sheet name="RIDE_REQUEST" sheetId="3" r:id="rId1"/>
     <sheet name="NPC_ID" sheetId="1" r:id="rId2"/>
-    <sheet name="LOCATION_POOL" sheetId="5" r:id="rId3"/>
+    <sheet name="LOCATION_ID" sheetId="5" r:id="rId3"/>
     <sheet name="DIALOGUE_POOL" sheetId="2" r:id="rId4"/>
-    <sheet name="DIAG_TITLE_POOL" sheetId="6" r:id="rId5"/>
+    <sheet name="TAGS" sheetId="7" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="NPC_IDs">NPC_ID!$A$2:$A$1048576</definedName>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="57">
   <si>
     <t>ID</t>
   </si>
@@ -105,18 +105,6 @@
     <t>jimmy.trust</t>
   </si>
   <si>
-    <t>hannah.neutral</t>
-  </si>
-  <si>
-    <t>jimmy.firstmet</t>
-  </si>
-  <si>
-    <t>jimmy. trust</t>
-  </si>
-  <si>
-    <t>TAG</t>
-  </si>
-  <si>
     <t>02</t>
   </si>
   <si>
@@ -153,59 +141,71 @@
     <t>006</t>
   </si>
   <si>
-    <t>001.transition</t>
-  </si>
-  <si>
-    <t>001.geton</t>
-  </si>
-  <si>
-    <t>001.during</t>
-  </si>
-  <si>
-    <t>001.end</t>
-  </si>
-  <si>
-    <t>002.transition</t>
-  </si>
-  <si>
-    <t>003.transition</t>
-  </si>
-  <si>
-    <t>004.transition</t>
-  </si>
-  <si>
-    <t>002.geton</t>
-  </si>
-  <si>
-    <t>003.geton</t>
-  </si>
-  <si>
-    <t>004.geton</t>
-  </si>
-  <si>
-    <t>002.during</t>
-  </si>
-  <si>
-    <t>003.during</t>
-  </si>
-  <si>
-    <t>004.during</t>
-  </si>
-  <si>
-    <t>002.end</t>
-  </si>
-  <si>
-    <t>003.end</t>
-  </si>
-  <si>
-    <t>004.end</t>
+    <t>HANNAH_MET</t>
+  </si>
+  <si>
+    <t>HANNAH_ALIVE</t>
+  </si>
+  <si>
+    <t>JIMMY_TRUSTS</t>
+  </si>
+  <si>
+    <t>DELIVERED_MESSAGE</t>
+  </si>
+  <si>
+    <t>World Event</t>
+  </si>
+  <si>
+    <t>Gameplay Tags</t>
+  </si>
+  <si>
+    <t>SHORTCUT_001</t>
+  </si>
+  <si>
+    <t>SHORTCUT_002</t>
+  </si>
+  <si>
+    <t>SHORTCUT_003</t>
+  </si>
+  <si>
+    <t>CORP_HIRING</t>
+  </si>
+  <si>
+    <t>yay</t>
+  </si>
+  <si>
+    <t>yo</t>
+  </si>
+  <si>
+    <t>SEGMENT</t>
+  </si>
+  <si>
+    <t>CONDITION</t>
+  </si>
+  <si>
+    <t>DAY</t>
+  </si>
+  <si>
+    <t>yar</t>
+  </si>
+  <si>
+    <t>yip</t>
+  </si>
+  <si>
+    <t>DAY_ONE</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>04</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -359,8 +359,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -538,6 +553,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -758,7 +779,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -803,6 +824,28 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1182,43 +1225,52 @@
   <dimension ref="A1:Y44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.5546875" style="4" customWidth="1"/>
-    <col min="2" max="6" width="12.6640625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" style="24" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="16.77734375" style="4" customWidth="1"/>
+    <col min="4" max="6" width="12.6640625" style="4" customWidth="1"/>
     <col min="7" max="7" width="16.33203125" style="4" customWidth="1"/>
-    <col min="8" max="10" width="12.6640625" style="8" customWidth="1"/>
-    <col min="11" max="25" width="9.109375" style="9"/>
+    <col min="8" max="8" width="12.6640625" style="8" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" style="8" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" style="8" customWidth="1"/>
+    <col min="11" max="11" width="16.109375" style="9" customWidth="1"/>
+    <col min="12" max="25" width="9.109375" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="1" customFormat="1" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
+      <c r="J1" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>50</v>
+      </c>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
       <c r="N1" s="6"/>
@@ -1234,36 +1286,40 @@
       <c r="X1" s="6"/>
       <c r="Y1" s="6"/>
     </row>
-    <row r="2" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:25" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="23">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="D2" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
+        <v>32</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>54</v>
+      </c>
       <c r="L2" s="4"/>
       <c r="M2" s="4"/>
       <c r="N2" s="4"/>
@@ -1279,35 +1335,37 @@
       <c r="X2" s="4"/>
       <c r="Y2" s="4"/>
     </row>
-    <row r="3" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:25" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="23">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="D3" s="4" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J3" s="4"/>
+        <v>32</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
@@ -1324,35 +1382,37 @@
       <c r="X3" s="4"/>
       <c r="Y3" s="4"/>
     </row>
-    <row r="4" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:25" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="23">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="D4" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J4" s="4"/>
+        <v>36</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
@@ -1369,35 +1429,37 @@
       <c r="X4" s="4"/>
       <c r="Y4" s="4"/>
     </row>
-    <row r="5" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:25" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="23">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>37</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>35</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J5" s="4"/>
+        <v>33</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
@@ -1415,6 +1477,8 @@
       <c r="Y5" s="4"/>
     </row>
     <row r="6" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="23"/>
+      <c r="B6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
@@ -1433,7 +1497,7 @@
       <c r="Y6" s="4"/>
     </row>
     <row r="7" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4"/>
+      <c r="A7" s="24"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
@@ -1460,7 +1524,7 @@
       <c r="Y7" s="4"/>
     </row>
     <row r="8" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4"/>
+      <c r="A8" s="24"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -1487,7 +1551,7 @@
       <c r="Y8" s="4"/>
     </row>
     <row r="9" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="4"/>
+      <c r="A9" s="24"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -1514,7 +1578,7 @@
       <c r="Y9" s="4"/>
     </row>
     <row r="10" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="4"/>
+      <c r="A10" s="24"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -1541,7 +1605,7 @@
       <c r="Y10" s="4"/>
     </row>
     <row r="11" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="4"/>
+      <c r="A11" s="24"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -1568,7 +1632,7 @@
       <c r="Y11" s="4"/>
     </row>
     <row r="12" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="4"/>
+      <c r="A12" s="24"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
@@ -1595,7 +1659,7 @@
       <c r="Y12" s="4"/>
     </row>
     <row r="13" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="4"/>
+      <c r="A13" s="24"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -1622,7 +1686,7 @@
       <c r="Y13" s="4"/>
     </row>
     <row r="14" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="4"/>
+      <c r="A14" s="24"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -1649,7 +1713,7 @@
       <c r="Y14" s="4"/>
     </row>
     <row r="15" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="4"/>
+      <c r="A15" s="24"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -1676,7 +1740,7 @@
       <c r="Y15" s="4"/>
     </row>
     <row r="16" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="4"/>
+      <c r="A16" s="24"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -1703,7 +1767,7 @@
       <c r="Y16" s="4"/>
     </row>
     <row r="17" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="4"/>
+      <c r="A17" s="24"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
@@ -1730,7 +1794,7 @@
       <c r="Y17" s="4"/>
     </row>
     <row r="18" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="4"/>
+      <c r="A18" s="24"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -1757,7 +1821,7 @@
       <c r="Y18" s="4"/>
     </row>
     <row r="19" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="4"/>
+      <c r="A19" s="24"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -1784,7 +1848,7 @@
       <c r="Y19" s="4"/>
     </row>
     <row r="20" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="4"/>
+      <c r="A20" s="24"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -1811,7 +1875,7 @@
       <c r="Y20" s="4"/>
     </row>
     <row r="21" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="4"/>
+      <c r="A21" s="24"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
@@ -1838,7 +1902,7 @@
       <c r="Y21" s="4"/>
     </row>
     <row r="22" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="4"/>
+      <c r="A22" s="24"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
@@ -1865,7 +1929,7 @@
       <c r="Y22" s="4"/>
     </row>
     <row r="23" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="4"/>
+      <c r="A23" s="24"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -1892,7 +1956,7 @@
       <c r="Y23" s="4"/>
     </row>
     <row r="24" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="4"/>
+      <c r="A24" s="24"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -1919,7 +1983,7 @@
       <c r="Y24" s="4"/>
     </row>
     <row r="25" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="4"/>
+      <c r="A25" s="24"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -1946,7 +2010,7 @@
       <c r="Y25" s="4"/>
     </row>
     <row r="26" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="4"/>
+      <c r="A26" s="24"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
@@ -1973,7 +2037,7 @@
       <c r="Y26" s="4"/>
     </row>
     <row r="27" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="4"/>
+      <c r="A27" s="24"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
@@ -2000,7 +2064,7 @@
       <c r="Y27" s="4"/>
     </row>
     <row r="28" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="4"/>
+      <c r="A28" s="24"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -2027,7 +2091,7 @@
       <c r="Y28" s="4"/>
     </row>
     <row r="29" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="4"/>
+      <c r="A29" s="24"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -2054,7 +2118,7 @@
       <c r="Y29" s="4"/>
     </row>
     <row r="30" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="4"/>
+      <c r="A30" s="24"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -2081,7 +2145,7 @@
       <c r="Y30" s="4"/>
     </row>
     <row r="31" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="4"/>
+      <c r="A31" s="24"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
@@ -2108,7 +2172,7 @@
       <c r="Y31" s="4"/>
     </row>
     <row r="32" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="4"/>
+      <c r="A32" s="24"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
@@ -2135,7 +2199,7 @@
       <c r="Y32" s="4"/>
     </row>
     <row r="33" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="4"/>
+      <c r="A33" s="24"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
@@ -2162,7 +2226,7 @@
       <c r="Y33" s="4"/>
     </row>
     <row r="34" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="4"/>
+      <c r="A34" s="24"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
@@ -2189,7 +2253,7 @@
       <c r="Y34" s="4"/>
     </row>
     <row r="35" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="4"/>
+      <c r="A35" s="24"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
@@ -2216,7 +2280,7 @@
       <c r="Y35" s="4"/>
     </row>
     <row r="36" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="4"/>
+      <c r="A36" s="24"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
@@ -2243,7 +2307,7 @@
       <c r="Y36" s="4"/>
     </row>
     <row r="37" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="4"/>
+      <c r="A37" s="24"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
@@ -2270,7 +2334,7 @@
       <c r="Y37" s="4"/>
     </row>
     <row r="38" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="4"/>
+      <c r="A38" s="24"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
@@ -2297,7 +2361,7 @@
       <c r="Y38" s="4"/>
     </row>
     <row r="39" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="4"/>
+      <c r="A39" s="24"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
@@ -2324,7 +2388,7 @@
       <c r="Y39" s="4"/>
     </row>
     <row r="40" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="4"/>
+      <c r="A40" s="24"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
@@ -2351,7 +2415,7 @@
       <c r="Y40" s="4"/>
     </row>
     <row r="41" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="4"/>
+      <c r="A41" s="24"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
@@ -2378,7 +2442,7 @@
       <c r="Y41" s="4"/>
     </row>
     <row r="42" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="4"/>
+      <c r="A42" s="24"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
@@ -2405,7 +2469,7 @@
       <c r="Y42" s="4"/>
     </row>
     <row r="43" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="4"/>
+      <c r="A43" s="24"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
@@ -2432,7 +2496,7 @@
       <c r="Y43" s="4"/>
     </row>
     <row r="44" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="4"/>
+      <c r="A44" s="24"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
@@ -2459,6 +2523,9 @@
       <c r="Y44" s="4"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B15">
+    <sortCondition descending="1" ref="B2:B15"/>
+  </sortState>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2485,10 +2552,10 @@
         <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -2516,13 +2583,13 @@
         <v>3</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
@@ -2550,13 +2617,13 @@
         <v>5</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
@@ -3497,7 +3564,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -3505,7 +3572,7 @@
         <v>11</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -3513,7 +3580,7 @@
         <v>12</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -3521,7 +3588,7 @@
         <v>13</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -3529,7 +3596,7 @@
         <v>14</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -3537,7 +3604,7 @@
         <v>15</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -3588,22 +3655,22 @@
     </row>
     <row r="2" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -3617,22 +3684,22 @@
     </row>
     <row r="3" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D3" s="15" t="s">
         <v>48</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -3646,22 +3713,22 @@
     </row>
     <row r="4" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
-        <v>26</v>
+        <v>52</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="F4" s="16" t="s">
-        <v>55</v>
+      <c r="F4" s="15" t="s">
+        <v>52</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -3675,22 +3742,22 @@
     </row>
     <row r="5" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E5" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="16" t="s">
-        <v>56</v>
+      <c r="F5" s="15" t="s">
+        <v>53</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -4084,10 +4151,102 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F566A316-34B4-4B5B-8946-6108E462BA0B}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63DF2F9F-84FB-4689-BEA6-08562272D65E}">
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13" style="22" customWidth="1"/>
+    <col min="2" max="2" width="26.88671875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" style="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="20"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+    </row>
+    <row r="2" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="21"/>
+      <c r="B3" s="19" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="21"/>
+      <c r="B5" s="19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="21"/>
+    </row>
+    <row r="8" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="21"/>
+    </row>
+    <row r="9" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="21"/>
+    </row>
+    <row r="10" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="21"/>
+      <c r="B11" s="19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="21"/>
+      <c r="B12" s="19" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+  </mergeCells>
+  <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Request assignment + spawn system
</commit_message>
<xml_diff>
--- a/Assets/Database/Database.xlsx
+++ b/Assets/Database/Database.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tqhie\Unity Projects\Where-To\Assets\Database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UnityProjects\Where-To\Assets\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967C552E-945C-43E2-A724-BA640711811B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{270F4F97-C53C-429B-B9C7-723F6BFCA5CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0E7384ED-7C35-4E8F-B735-540A4F72621F}"/>
+    <workbookView xWindow="0" yWindow="2565" windowWidth="21600" windowHeight="11295" xr2:uid="{0E7384ED-7C35-4E8F-B735-540A4F72621F}"/>
   </bookViews>
   <sheets>
     <sheet name="RIDE_REQUEST" sheetId="3" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="73">
   <si>
     <t>ID</t>
   </si>
@@ -248,6 +248,18 @@
   </si>
   <si>
     <t>008</t>
+  </si>
+  <si>
+    <t>05</t>
+  </si>
+  <si>
+    <t>06</t>
+  </si>
+  <si>
+    <t>07</t>
+  </si>
+  <si>
+    <t>08</t>
   </si>
 </sst>
 </file>
@@ -1043,140 +1055,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -1320,6 +1198,140 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1339,39 +1351,39 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{161AE955-486A-4B61-AB78-C3AA8F8B1EE3}" name="Npc_Pool" displayName="Npc_Pool" ref="A1:D1048576" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{161AE955-486A-4B61-AB78-C3AA8F8B1EE3}" name="Npc_Pool" displayName="Npc_Pool" ref="A1:D1048576" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="A1:D1048576" xr:uid="{161AE955-486A-4B61-AB78-C3AA8F8B1EE3}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{971E0D76-6A3F-4CF4-9277-48BF668D7B2A}" name="NAME" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{D8546E7C-877C-4F1C-8E73-97DC7FF6C2E4}" name="ID" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{CF298EB9-7166-442D-A8F6-94DABD83C499}" name="DISPLAY NAME" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{87607142-5392-4BB1-B1D7-AB5BF175E58C}" name="MODEL" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{971E0D76-6A3F-4CF4-9277-48BF668D7B2A}" name="NAME" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{D8546E7C-877C-4F1C-8E73-97DC7FF6C2E4}" name="ID" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{CF298EB9-7166-442D-A8F6-94DABD83C499}" name="DISPLAY NAME" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{87607142-5392-4BB1-B1D7-AB5BF175E58C}" name="MODEL" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{5F401D05-9421-4373-910E-DBBA5D979DE7}" name="Location_Pool" displayName="Location_Pool" ref="A1:B1048576" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{5F401D05-9421-4373-910E-DBBA5D979DE7}" name="Location_Pool" displayName="Location_Pool" ref="A1:B1048576" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
   <autoFilter ref="A1:B1048576" xr:uid="{5F401D05-9421-4373-910E-DBBA5D979DE7}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{341D5880-1BC7-443E-84D3-F7E4F845AABB}" name="NAME" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{4AC38A0B-F596-43AE-9D82-EF556B360AD3}" name="ID" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{341D5880-1BC7-443E-84D3-F7E4F845AABB}" name="NAME" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{4AC38A0B-F596-43AE-9D82-EF556B360AD3}" name="ID" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{92921925-D6AA-4E7D-9EAD-225A1668D079}" name="Dialogue_Pool" displayName="Dialogue_Pool" ref="A1:F1048576" totalsRowShown="0" headerRowDxfId="23" dataDxfId="21" headerRowBorderDxfId="22" tableBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{92921925-D6AA-4E7D-9EAD-225A1668D079}" name="Dialogue_Pool" displayName="Dialogue_Pool" ref="A1:F1048576" totalsRowShown="0" headerRowDxfId="13" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10">
   <autoFilter ref="A1:F1048576" xr:uid="{92921925-D6AA-4E7D-9EAD-225A1668D079}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{3F3F7530-7538-4241-8E3F-F27878961117}" name="NAME" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{1E0CD6DB-3A7B-4CC8-9D99-7EA296CB5FF7}" name="ID" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{DE87D127-4E31-4D1A-9888-EC481693215F}" name="TRANSITION" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{9C47E7D4-77BE-467D-B61D-7CF4316A873D}" name="GETON " dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{94EED148-A6FE-4682-8419-11F273DC0FAC}" name="END" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{CF0ECC79-0238-470B-AE20-AE227DD1944E}" name="DURING" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{3F3F7530-7538-4241-8E3F-F27878961117}" name="NAME" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{1E0CD6DB-3A7B-4CC8-9D99-7EA296CB5FF7}" name="ID" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{DE87D127-4E31-4D1A-9888-EC481693215F}" name="TRANSITION" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{9C47E7D4-77BE-467D-B61D-7CF4316A873D}" name="GETON " dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{94EED148-A6FE-4682-8419-11F273DC0FAC}" name="END" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{CF0ECC79-0238-470B-AE20-AE227DD1944E}" name="DURING" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1706,21 +1718,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{847982F6-4584-4784-B812-EAA01FCD0B25}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Z44"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.5546875" style="15" customWidth="1"/>
-    <col min="2" max="2" width="18.88671875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="11.44140625" style="3" customWidth="1"/>
-    <col min="4" max="6" width="12.6640625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" style="3" customWidth="1"/>
-    <col min="10" max="10" width="13.77734375" style="7" customWidth="1"/>
-    <col min="11" max="11" width="15.6640625" style="7" customWidth="1"/>
-    <col min="18" max="26" width="9.109375" style="8"/>
+    <col min="1" max="1" width="17.5703125" style="15" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" style="3" customWidth="1"/>
+    <col min="4" max="6" width="12.7109375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" style="3" customWidth="1"/>
+    <col min="9" max="9" width="16.28515625" style="3" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" style="7" customWidth="1"/>
+    <col min="18" max="26" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="1" customFormat="1" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" s="1" customFormat="1" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
@@ -1764,7 +1776,7 @@
       <c r="Y1" s="5"/>
       <c r="Z1" s="5"/>
     </row>
-    <row r="2" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12">
         <v>1</v>
       </c>
@@ -1808,7 +1820,7 @@
       <c r="Y2" s="3"/>
       <c r="Z2" s="3"/>
     </row>
-    <row r="3" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12">
         <v>1</v>
       </c>
@@ -1819,7 +1831,7 @@
         <v>21</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>64</v>
@@ -1852,7 +1864,7 @@
       <c r="Y3" s="3"/>
       <c r="Z3" s="3"/>
     </row>
-    <row r="4" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -1863,7 +1875,7 @@
         <v>24</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>65</v>
@@ -1896,7 +1908,7 @@
       <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
     </row>
-    <row r="5" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>1</v>
       </c>
@@ -1907,7 +1919,7 @@
         <v>25</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>66</v>
@@ -1940,7 +1952,7 @@
       <c r="Y5" s="3"/>
       <c r="Z5" s="3"/>
     </row>
-    <row r="6" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>1</v>
       </c>
@@ -1951,7 +1963,7 @@
         <v>23</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>63</v>
@@ -1984,7 +1996,7 @@
       <c r="Y6" s="3"/>
       <c r="Z6" s="3"/>
     </row>
-    <row r="7" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>1</v>
       </c>
@@ -1995,7 +2007,7 @@
         <v>26</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>64</v>
@@ -2028,7 +2040,7 @@
       <c r="Y7" s="3"/>
       <c r="Z7" s="3"/>
     </row>
-    <row r="8" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>1</v>
       </c>
@@ -2039,7 +2051,7 @@
         <v>67</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>65</v>
@@ -2072,7 +2084,7 @@
       <c r="Y8" s="3"/>
       <c r="Z8" s="3"/>
     </row>
-    <row r="9" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="12">
         <v>1</v>
       </c>
@@ -2083,7 +2095,7 @@
         <v>68</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>66</v>
@@ -2116,7 +2128,7 @@
       <c r="Y9" s="3"/>
       <c r="Z9" s="3"/>
     </row>
-    <row r="10" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -2138,7 +2150,7 @@
       <c r="Y10" s="3"/>
       <c r="Z10" s="3"/>
     </row>
-    <row r="11" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -2160,7 +2172,7 @@
       <c r="Y11" s="3"/>
       <c r="Z11" s="3"/>
     </row>
-    <row r="12" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="15"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -2182,7 +2194,7 @@
       <c r="Y12" s="3"/>
       <c r="Z12" s="3"/>
     </row>
-    <row r="13" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="15"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -2204,7 +2216,7 @@
       <c r="Y13" s="3"/>
       <c r="Z13" s="3"/>
     </row>
-    <row r="14" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="15"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -2226,7 +2238,7 @@
       <c r="Y14" s="3"/>
       <c r="Z14" s="3"/>
     </row>
-    <row r="15" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -2248,7 +2260,7 @@
       <c r="Y15" s="3"/>
       <c r="Z15" s="3"/>
     </row>
-    <row r="16" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="15"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -2270,7 +2282,7 @@
       <c r="Y16" s="3"/>
       <c r="Z16" s="3"/>
     </row>
-    <row r="17" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="15"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -2292,7 +2304,7 @@
       <c r="Y17" s="3"/>
       <c r="Z17" s="3"/>
     </row>
-    <row r="18" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="15"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -2314,7 +2326,7 @@
       <c r="Y18" s="3"/>
       <c r="Z18" s="3"/>
     </row>
-    <row r="19" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="15"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -2336,7 +2348,7 @@
       <c r="Y19" s="3"/>
       <c r="Z19" s="3"/>
     </row>
-    <row r="20" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="15"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -2358,7 +2370,7 @@
       <c r="Y20" s="3"/>
       <c r="Z20" s="3"/>
     </row>
-    <row r="21" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="15"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -2380,7 +2392,7 @@
       <c r="Y21" s="3"/>
       <c r="Z21" s="3"/>
     </row>
-    <row r="22" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="15"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -2402,7 +2414,7 @@
       <c r="Y22" s="3"/>
       <c r="Z22" s="3"/>
     </row>
-    <row r="23" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="15"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -2424,7 +2436,7 @@
       <c r="Y23" s="3"/>
       <c r="Z23" s="3"/>
     </row>
-    <row r="24" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="15"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -2446,7 +2458,7 @@
       <c r="Y24" s="3"/>
       <c r="Z24" s="3"/>
     </row>
-    <row r="25" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="15"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -2468,7 +2480,7 @@
       <c r="Y25" s="3"/>
       <c r="Z25" s="3"/>
     </row>
-    <row r="26" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="15"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -2490,7 +2502,7 @@
       <c r="Y26" s="3"/>
       <c r="Z26" s="3"/>
     </row>
-    <row r="27" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="15"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -2512,7 +2524,7 @@
       <c r="Y27" s="3"/>
       <c r="Z27" s="3"/>
     </row>
-    <row r="28" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="15"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -2534,7 +2546,7 @@
       <c r="Y28" s="3"/>
       <c r="Z28" s="3"/>
     </row>
-    <row r="29" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="15"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -2556,7 +2568,7 @@
       <c r="Y29" s="3"/>
       <c r="Z29" s="3"/>
     </row>
-    <row r="30" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="15"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -2578,7 +2590,7 @@
       <c r="Y30" s="3"/>
       <c r="Z30" s="3"/>
     </row>
-    <row r="31" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="15"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -2600,7 +2612,7 @@
       <c r="Y31" s="3"/>
       <c r="Z31" s="3"/>
     </row>
-    <row r="32" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="15"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -2622,7 +2634,7 @@
       <c r="Y32" s="3"/>
       <c r="Z32" s="3"/>
     </row>
-    <row r="33" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="15"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -2644,7 +2656,7 @@
       <c r="Y33" s="3"/>
       <c r="Z33" s="3"/>
     </row>
-    <row r="34" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -2666,7 +2678,7 @@
       <c r="Y34" s="3"/>
       <c r="Z34" s="3"/>
     </row>
-    <row r="35" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="15"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -2688,7 +2700,7 @@
       <c r="Y35" s="3"/>
       <c r="Z35" s="3"/>
     </row>
-    <row r="36" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="15"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -2710,7 +2722,7 @@
       <c r="Y36" s="3"/>
       <c r="Z36" s="3"/>
     </row>
-    <row r="37" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="15"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -2732,7 +2744,7 @@
       <c r="Y37" s="3"/>
       <c r="Z37" s="3"/>
     </row>
-    <row r="38" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="15"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -2754,7 +2766,7 @@
       <c r="Y38" s="3"/>
       <c r="Z38" s="3"/>
     </row>
-    <row r="39" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="15"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -2776,7 +2788,7 @@
       <c r="Y39" s="3"/>
       <c r="Z39" s="3"/>
     </row>
-    <row r="40" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="15"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -2798,7 +2810,7 @@
       <c r="Y40" s="3"/>
       <c r="Z40" s="3"/>
     </row>
-    <row r="41" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="15"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -2820,7 +2832,7 @@
       <c r="Y41" s="3"/>
       <c r="Z41" s="3"/>
     </row>
-    <row r="42" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="15"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -2842,7 +2854,7 @@
       <c r="Y42" s="3"/>
       <c r="Z42" s="3"/>
     </row>
-    <row r="43" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="15"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -2864,7 +2876,7 @@
       <c r="Y43" s="3"/>
       <c r="Z43" s="3"/>
     </row>
-    <row r="44" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="15"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -2916,17 +2928,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B698B908-9440-4773-9B30-11BAE7A1734C}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:X37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.33203125" style="9" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" style="9" customWidth="1"/>
-    <col min="3" max="3" width="24.109375" style="9" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" style="3" customWidth="1"/>
-    <col min="5" max="16" width="9.109375" style="3"/>
-    <col min="17" max="24" width="9.109375" style="8"/>
+    <col min="1" max="1" width="24.28515625" style="9" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="24.140625" style="9" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" style="3" customWidth="1"/>
+    <col min="5" max="16" width="9.140625" style="3"/>
+    <col min="17" max="24" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>2</v>
       </c>
@@ -2960,7 +2972,7 @@
       <c r="W1" s="5"/>
       <c r="X1" s="5"/>
     </row>
-    <row r="2" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>3</v>
       </c>
@@ -2994,7 +3006,7 @@
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
     </row>
-    <row r="3" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>5</v>
       </c>
@@ -3028,7 +3040,7 @@
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
     </row>
-    <row r="4" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9"/>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
@@ -3054,7 +3066,7 @@
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
     </row>
-    <row r="5" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -3080,7 +3092,7 @@
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
     </row>
-    <row r="6" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -3106,7 +3118,7 @@
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
     </row>
-    <row r="7" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -3132,7 +3144,7 @@
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
     </row>
-    <row r="8" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -3158,7 +3170,7 @@
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
     </row>
-    <row r="9" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -3184,7 +3196,7 @@
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
     </row>
-    <row r="10" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -3210,7 +3222,7 @@
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
     </row>
-    <row r="11" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -3236,7 +3248,7 @@
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
     </row>
-    <row r="12" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -3262,7 +3274,7 @@
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
     </row>
-    <row r="13" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -3288,7 +3300,7 @@
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
     </row>
-    <row r="14" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -3314,7 +3326,7 @@
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
     </row>
-    <row r="15" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -3340,7 +3352,7 @@
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
     </row>
-    <row r="16" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9"/>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -3366,7 +3378,7 @@
       <c r="W16" s="3"/>
       <c r="X16" s="3"/>
     </row>
-    <row r="17" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -3392,7 +3404,7 @@
       <c r="W17" s="3"/>
       <c r="X17" s="3"/>
     </row>
-    <row r="18" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -3418,7 +3430,7 @@
       <c r="W18" s="3"/>
       <c r="X18" s="3"/>
     </row>
-    <row r="19" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
@@ -3444,7 +3456,7 @@
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
     </row>
-    <row r="20" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -3470,7 +3482,7 @@
       <c r="W20" s="3"/>
       <c r="X20" s="3"/>
     </row>
-    <row r="21" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9"/>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
@@ -3496,7 +3508,7 @@
       <c r="W21" s="3"/>
       <c r="X21" s="3"/>
     </row>
-    <row r="22" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
@@ -3522,7 +3534,7 @@
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
     </row>
-    <row r="23" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
@@ -3548,7 +3560,7 @@
       <c r="W23" s="3"/>
       <c r="X23" s="3"/>
     </row>
-    <row r="24" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9"/>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
@@ -3574,7 +3586,7 @@
       <c r="W24" s="3"/>
       <c r="X24" s="3"/>
     </row>
-    <row r="25" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9"/>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
@@ -3600,7 +3612,7 @@
       <c r="W25" s="3"/>
       <c r="X25" s="3"/>
     </row>
-    <row r="26" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -3626,7 +3638,7 @@
       <c r="W26" s="3"/>
       <c r="X26" s="3"/>
     </row>
-    <row r="27" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="9"/>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
@@ -3652,7 +3664,7 @@
       <c r="W27" s="3"/>
       <c r="X27" s="3"/>
     </row>
-    <row r="28" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9"/>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -3678,7 +3690,7 @@
       <c r="W28" s="3"/>
       <c r="X28" s="3"/>
     </row>
-    <row r="29" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="9"/>
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
@@ -3704,7 +3716,7 @@
       <c r="W29" s="3"/>
       <c r="X29" s="3"/>
     </row>
-    <row r="30" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -3730,7 +3742,7 @@
       <c r="W30" s="3"/>
       <c r="X30" s="3"/>
     </row>
-    <row r="31" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="9"/>
       <c r="B31" s="9"/>
       <c r="C31" s="9"/>
@@ -3756,7 +3768,7 @@
       <c r="W31" s="3"/>
       <c r="X31" s="3"/>
     </row>
-    <row r="32" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="9"/>
       <c r="B32" s="9"/>
       <c r="C32" s="9"/>
@@ -3782,7 +3794,7 @@
       <c r="W32" s="3"/>
       <c r="X32" s="3"/>
     </row>
-    <row r="33" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="9"/>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
@@ -3808,7 +3820,7 @@
       <c r="W33" s="3"/>
       <c r="X33" s="3"/>
     </row>
-    <row r="34" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -3834,7 +3846,7 @@
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
     </row>
-    <row r="35" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="9"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -3860,7 +3872,7 @@
       <c r="W35" s="3"/>
       <c r="X35" s="3"/>
     </row>
-    <row r="36" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="9"/>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
@@ -3886,7 +3898,7 @@
       <c r="W36" s="3"/>
       <c r="X36" s="3"/>
     </row>
-    <row r="37" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="9"/>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
@@ -3929,14 +3941,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EE75206-B358-44F7-8367-AB97E19840D2}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AA7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="17.33203125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" style="8" customWidth="1"/>
-    <col min="4" max="27" width="9.109375" style="8"/>
+    <col min="1" max="2" width="17.28515625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" style="8" customWidth="1"/>
+    <col min="4" max="27" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>2</v>
       </c>
@@ -3945,7 +3957,7 @@
       </c>
       <c r="C1" s="6"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -3953,7 +3965,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -3961,7 +3973,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -3969,7 +3981,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
@@ -3977,7 +3989,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -3985,7 +3997,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
@@ -4006,16 +4018,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E3F026-F201-4063-9685-60C58AB78B27}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="23" customWidth="1"/>
-    <col min="2" max="2" width="8.88671875" style="20"/>
+    <col min="1" max="1" width="8.85546875" style="23" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" style="20"/>
     <col min="3" max="5" width="27" style="20" customWidth="1"/>
     <col min="6" max="6" width="27" style="26" customWidth="1"/>
     <col min="7" max="7" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="16" customFormat="1" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" s="16" customFormat="1" ht="22.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>2</v>
       </c>
@@ -4040,7 +4052,7 @@
       <c r="J1" s="5"/>
       <c r="K1" s="5"/>
     </row>
-    <row r="2" spans="1:11" s="17" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" s="17" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
         <v>36</v>
       </c>
@@ -4060,7 +4072,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="22" t="s">
         <v>37</v>
       </c>
@@ -4080,7 +4092,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
         <v>41</v>
       </c>
@@ -4100,7 +4112,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="22" t="s">
         <v>42</v>
       </c>
@@ -4145,14 +4157,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63DF2F9F-84FB-4689-BEA6-08562272D65E}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:L13"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" style="14" customWidth="1"/>
-    <col min="2" max="2" width="26.88671875" style="12" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="12"/>
+    <col min="2" max="2" width="26.85546875" style="12" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="13"/>
       <c r="B1" s="30" t="s">
         <v>60</v>
@@ -4165,7 +4177,7 @@
       <c r="H1" s="10"/>
       <c r="I1" s="10"/>
     </row>
-    <row r="2" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="31" t="s">
         <v>31</v>
       </c>
@@ -4173,13 +4185,13 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31"/>
       <c r="B3" s="12" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="31"/>
       <c r="B4" s="12" t="s">
         <v>46</v>
@@ -4188,10 +4200,10 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="31"/>
     </row>
-    <row r="6" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="s">
         <v>32</v>
       </c>
@@ -4199,25 +4211,25 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="31"/>
       <c r="B7" s="12" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="31"/>
       <c r="B8" s="12" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="31"/>
       <c r="B9" s="12" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="31" t="s">
         <v>1</v>
       </c>
@@ -4225,13 +4237,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="31"/>
       <c r="B11" s="12" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="31" t="s">
         <v>4</v>
       </c>
@@ -4239,7 +4251,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="31"/>
       <c r="B13" s="12" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Pickup + Database merge WIP
</commit_message>
<xml_diff>
--- a/Assets/Database/Database.xlsx
+++ b/Assets/Database/Database.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UnityProjects\Where-To\Assets\Database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tqhie\Unity Projects\Where-To\Assets\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{270F4F97-C53C-429B-B9C7-723F6BFCA5CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFD0C729-E1C6-4982-B2D5-CB2E69B4F8D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2565" windowWidth="21600" windowHeight="11295" xr2:uid="{0E7384ED-7C35-4E8F-B735-540A4F72621F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0E7384ED-7C35-4E8F-B735-540A4F72621F}"/>
   </bookViews>
   <sheets>
     <sheet name="RIDE_REQUEST" sheetId="3" r:id="rId1"/>
@@ -184,18 +184,6 @@
     <t>HEY</t>
   </si>
   <si>
-    <t>zero.one</t>
-  </si>
-  <si>
-    <t>zero.two</t>
-  </si>
-  <si>
-    <t>zero.three</t>
-  </si>
-  <si>
-    <t>zero.four</t>
-  </si>
-  <si>
     <t>S</t>
   </si>
   <si>
@@ -250,16 +238,28 @@
     <t>008</t>
   </si>
   <si>
-    <t>05</t>
-  </si>
-  <si>
-    <t>06</t>
-  </si>
-  <si>
-    <t>07</t>
-  </si>
-  <si>
-    <t>08</t>
+    <t>one</t>
+  </si>
+  <si>
+    <t>two</t>
+  </si>
+  <si>
+    <t>three</t>
+  </si>
+  <si>
+    <t>four</t>
+  </si>
+  <si>
+    <t>five</t>
+  </si>
+  <si>
+    <t>six</t>
+  </si>
+  <si>
+    <t>eight</t>
+  </si>
+  <si>
+    <t>seven</t>
   </si>
 </sst>
 </file>
@@ -1718,21 +1718,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{847982F6-4584-4784-B812-EAA01FCD0B25}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Z44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" style="15" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="3" customWidth="1"/>
-    <col min="4" max="6" width="12.7109375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" style="3" customWidth="1"/>
-    <col min="9" max="9" width="16.28515625" style="3" customWidth="1"/>
-    <col min="10" max="10" width="13.7109375" style="7" customWidth="1"/>
-    <col min="11" max="11" width="15.7109375" style="7" customWidth="1"/>
-    <col min="18" max="26" width="9.140625" style="8"/>
+    <col min="1" max="1" width="17.5546875" style="15" customWidth="1"/>
+    <col min="2" max="2" width="18.88671875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" style="3" customWidth="1"/>
+    <col min="4" max="6" width="12.6640625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="13.6640625" style="7" customWidth="1"/>
+    <col min="11" max="11" width="15.6640625" style="7" customWidth="1"/>
+    <col min="18" max="26" width="9.109375" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="1" customFormat="1" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" s="1" customFormat="1" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
@@ -1746,7 +1746,7 @@
         <v>38</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>6</v>
@@ -1776,21 +1776,21 @@
       <c r="Y1" s="5"/>
       <c r="Z1" s="5"/>
     </row>
-    <row r="2" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="12">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>22</v>
@@ -1820,21 +1820,21 @@
       <c r="Y2" s="3"/>
       <c r="Z2" s="3"/>
     </row>
-    <row r="3" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="12">
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>21</v>
@@ -1852,7 +1852,7 @@
         <v>14</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="R3" s="3"/>
       <c r="S3" s="3"/>
@@ -1864,21 +1864,21 @@
       <c r="Y3" s="3"/>
       <c r="Z3" s="3"/>
     </row>
-    <row r="4" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>24</v>
@@ -1908,21 +1908,21 @@
       <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
     </row>
-    <row r="5" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>1</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>25</v>
@@ -1940,7 +1940,7 @@
         <v>10</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -1952,21 +1952,21 @@
       <c r="Y5" s="3"/>
       <c r="Z5" s="3"/>
     </row>
-    <row r="6" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>1</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>22</v>
@@ -1996,21 +1996,21 @@
       <c r="Y6" s="3"/>
       <c r="Z6" s="3"/>
     </row>
-    <row r="7" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>1</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>26</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>21</v>
@@ -2028,7 +2028,7 @@
         <v>14</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
@@ -2040,21 +2040,21 @@
       <c r="Y7" s="3"/>
       <c r="Z7" s="3"/>
     </row>
-    <row r="8" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="12">
         <v>1</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>24</v>
@@ -2084,21 +2084,21 @@
       <c r="Y8" s="3"/>
       <c r="Z8" s="3"/>
     </row>
-    <row r="9" spans="1:26" s="2" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" s="2" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="12">
         <v>1</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>25</v>
@@ -2116,7 +2116,7 @@
         <v>10</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
@@ -2128,7 +2128,7 @@
       <c r="Y9" s="3"/>
       <c r="Z9" s="3"/>
     </row>
-    <row r="10" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="15"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -2150,7 +2150,7 @@
       <c r="Y10" s="3"/>
       <c r="Z10" s="3"/>
     </row>
-    <row r="11" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="15"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -2172,7 +2172,7 @@
       <c r="Y11" s="3"/>
       <c r="Z11" s="3"/>
     </row>
-    <row r="12" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="15"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -2194,7 +2194,7 @@
       <c r="Y12" s="3"/>
       <c r="Z12" s="3"/>
     </row>
-    <row r="13" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="15"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -2216,7 +2216,7 @@
       <c r="Y13" s="3"/>
       <c r="Z13" s="3"/>
     </row>
-    <row r="14" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="15"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -2238,7 +2238,7 @@
       <c r="Y14" s="3"/>
       <c r="Z14" s="3"/>
     </row>
-    <row r="15" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="15"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -2260,7 +2260,7 @@
       <c r="Y15" s="3"/>
       <c r="Z15" s="3"/>
     </row>
-    <row r="16" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="15"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -2282,7 +2282,7 @@
       <c r="Y16" s="3"/>
       <c r="Z16" s="3"/>
     </row>
-    <row r="17" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="15"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -2304,7 +2304,7 @@
       <c r="Y17" s="3"/>
       <c r="Z17" s="3"/>
     </row>
-    <row r="18" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="15"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -2326,7 +2326,7 @@
       <c r="Y18" s="3"/>
       <c r="Z18" s="3"/>
     </row>
-    <row r="19" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="15"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -2348,7 +2348,7 @@
       <c r="Y19" s="3"/>
       <c r="Z19" s="3"/>
     </row>
-    <row r="20" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="15"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -2370,7 +2370,7 @@
       <c r="Y20" s="3"/>
       <c r="Z20" s="3"/>
     </row>
-    <row r="21" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="15"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -2392,7 +2392,7 @@
       <c r="Y21" s="3"/>
       <c r="Z21" s="3"/>
     </row>
-    <row r="22" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="15"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -2414,7 +2414,7 @@
       <c r="Y22" s="3"/>
       <c r="Z22" s="3"/>
     </row>
-    <row r="23" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="15"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -2436,7 +2436,7 @@
       <c r="Y23" s="3"/>
       <c r="Z23" s="3"/>
     </row>
-    <row r="24" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="15"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -2458,7 +2458,7 @@
       <c r="Y24" s="3"/>
       <c r="Z24" s="3"/>
     </row>
-    <row r="25" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="15"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -2480,7 +2480,7 @@
       <c r="Y25" s="3"/>
       <c r="Z25" s="3"/>
     </row>
-    <row r="26" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="15"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -2502,7 +2502,7 @@
       <c r="Y26" s="3"/>
       <c r="Z26" s="3"/>
     </row>
-    <row r="27" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="15"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -2524,7 +2524,7 @@
       <c r="Y27" s="3"/>
       <c r="Z27" s="3"/>
     </row>
-    <row r="28" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="15"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -2546,7 +2546,7 @@
       <c r="Y28" s="3"/>
       <c r="Z28" s="3"/>
     </row>
-    <row r="29" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="15"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -2568,7 +2568,7 @@
       <c r="Y29" s="3"/>
       <c r="Z29" s="3"/>
     </row>
-    <row r="30" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="15"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -2590,7 +2590,7 @@
       <c r="Y30" s="3"/>
       <c r="Z30" s="3"/>
     </row>
-    <row r="31" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="15"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -2612,7 +2612,7 @@
       <c r="Y31" s="3"/>
       <c r="Z31" s="3"/>
     </row>
-    <row r="32" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="15"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -2634,7 +2634,7 @@
       <c r="Y32" s="3"/>
       <c r="Z32" s="3"/>
     </row>
-    <row r="33" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="15"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -2656,7 +2656,7 @@
       <c r="Y33" s="3"/>
       <c r="Z33" s="3"/>
     </row>
-    <row r="34" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="15"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -2678,7 +2678,7 @@
       <c r="Y34" s="3"/>
       <c r="Z34" s="3"/>
     </row>
-    <row r="35" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="15"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -2700,7 +2700,7 @@
       <c r="Y35" s="3"/>
       <c r="Z35" s="3"/>
     </row>
-    <row r="36" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="15"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -2722,7 +2722,7 @@
       <c r="Y36" s="3"/>
       <c r="Z36" s="3"/>
     </row>
-    <row r="37" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="15"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -2744,7 +2744,7 @@
       <c r="Y37" s="3"/>
       <c r="Z37" s="3"/>
     </row>
-    <row r="38" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="15"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -2766,7 +2766,7 @@
       <c r="Y38" s="3"/>
       <c r="Z38" s="3"/>
     </row>
-    <row r="39" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="15"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -2788,7 +2788,7 @@
       <c r="Y39" s="3"/>
       <c r="Z39" s="3"/>
     </row>
-    <row r="40" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="15"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -2810,7 +2810,7 @@
       <c r="Y40" s="3"/>
       <c r="Z40" s="3"/>
     </row>
-    <row r="41" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="15"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -2832,7 +2832,7 @@
       <c r="Y41" s="3"/>
       <c r="Z41" s="3"/>
     </row>
-    <row r="42" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="15"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -2854,7 +2854,7 @@
       <c r="Y42" s="3"/>
       <c r="Z42" s="3"/>
     </row>
-    <row r="43" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="15"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -2876,7 +2876,7 @@
       <c r="Y43" s="3"/>
       <c r="Z43" s="3"/>
     </row>
-    <row r="44" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="15"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -2928,17 +2928,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B698B908-9440-4773-9B30-11BAE7A1734C}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:X37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.28515625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="24.140625" style="9" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" style="3" customWidth="1"/>
-    <col min="5" max="16" width="9.140625" style="3"/>
-    <col min="17" max="24" width="9.140625" style="8"/>
+    <col min="1" max="1" width="24.33203125" style="9" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="24.109375" style="9" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" style="3" customWidth="1"/>
+    <col min="5" max="16" width="9.109375" style="3"/>
+    <col min="17" max="24" width="9.109375" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>2</v>
       </c>
@@ -2972,7 +2972,7 @@
       <c r="W1" s="5"/>
       <c r="X1" s="5"/>
     </row>
-    <row r="2" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>3</v>
       </c>
@@ -3006,7 +3006,7 @@
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
     </row>
-    <row r="3" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>5</v>
       </c>
@@ -3040,7 +3040,7 @@
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
     </row>
-    <row r="4" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9"/>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
@@ -3066,7 +3066,7 @@
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
     </row>
-    <row r="5" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -3092,7 +3092,7 @@
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
     </row>
-    <row r="6" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -3118,7 +3118,7 @@
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
     </row>
-    <row r="7" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -3144,7 +3144,7 @@
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
     </row>
-    <row r="8" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -3170,7 +3170,7 @@
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
     </row>
-    <row r="9" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -3196,7 +3196,7 @@
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
     </row>
-    <row r="10" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -3222,7 +3222,7 @@
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
     </row>
-    <row r="11" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -3248,7 +3248,7 @@
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
     </row>
-    <row r="12" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -3274,7 +3274,7 @@
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
     </row>
-    <row r="13" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="9"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -3300,7 +3300,7 @@
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
     </row>
-    <row r="14" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="9"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -3326,7 +3326,7 @@
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
     </row>
-    <row r="15" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="9"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -3352,7 +3352,7 @@
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
     </row>
-    <row r="16" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="9"/>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -3378,7 +3378,7 @@
       <c r="W16" s="3"/>
       <c r="X16" s="3"/>
     </row>
-    <row r="17" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="9"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -3404,7 +3404,7 @@
       <c r="W17" s="3"/>
       <c r="X17" s="3"/>
     </row>
-    <row r="18" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -3430,7 +3430,7 @@
       <c r="W18" s="3"/>
       <c r="X18" s="3"/>
     </row>
-    <row r="19" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
@@ -3456,7 +3456,7 @@
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
     </row>
-    <row r="20" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -3482,7 +3482,7 @@
       <c r="W20" s="3"/>
       <c r="X20" s="3"/>
     </row>
-    <row r="21" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="9"/>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
@@ -3508,7 +3508,7 @@
       <c r="W21" s="3"/>
       <c r="X21" s="3"/>
     </row>
-    <row r="22" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="9"/>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
@@ -3534,7 +3534,7 @@
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
     </row>
-    <row r="23" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
@@ -3560,7 +3560,7 @@
       <c r="W23" s="3"/>
       <c r="X23" s="3"/>
     </row>
-    <row r="24" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="9"/>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
@@ -3586,7 +3586,7 @@
       <c r="W24" s="3"/>
       <c r="X24" s="3"/>
     </row>
-    <row r="25" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="9"/>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
@@ -3612,7 +3612,7 @@
       <c r="W25" s="3"/>
       <c r="X25" s="3"/>
     </row>
-    <row r="26" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -3638,7 +3638,7 @@
       <c r="W26" s="3"/>
       <c r="X26" s="3"/>
     </row>
-    <row r="27" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9"/>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
@@ -3664,7 +3664,7 @@
       <c r="W27" s="3"/>
       <c r="X27" s="3"/>
     </row>
-    <row r="28" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9"/>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -3690,7 +3690,7 @@
       <c r="W28" s="3"/>
       <c r="X28" s="3"/>
     </row>
-    <row r="29" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9"/>
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
@@ -3716,7 +3716,7 @@
       <c r="W29" s="3"/>
       <c r="X29" s="3"/>
     </row>
-    <row r="30" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -3742,7 +3742,7 @@
       <c r="W30" s="3"/>
       <c r="X30" s="3"/>
     </row>
-    <row r="31" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="9"/>
       <c r="B31" s="9"/>
       <c r="C31" s="9"/>
@@ -3768,7 +3768,7 @@
       <c r="W31" s="3"/>
       <c r="X31" s="3"/>
     </row>
-    <row r="32" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="9"/>
       <c r="B32" s="9"/>
       <c r="C32" s="9"/>
@@ -3794,7 +3794,7 @@
       <c r="W32" s="3"/>
       <c r="X32" s="3"/>
     </row>
-    <row r="33" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="9"/>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
@@ -3820,7 +3820,7 @@
       <c r="W33" s="3"/>
       <c r="X33" s="3"/>
     </row>
-    <row r="34" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -3846,7 +3846,7 @@
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
     </row>
-    <row r="35" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="9"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -3872,7 +3872,7 @@
       <c r="W35" s="3"/>
       <c r="X35" s="3"/>
     </row>
-    <row r="36" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9"/>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
@@ -3898,7 +3898,7 @@
       <c r="W36" s="3"/>
       <c r="X36" s="3"/>
     </row>
-    <row r="37" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="9"/>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
@@ -3941,14 +3941,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EE75206-B358-44F7-8367-AB97E19840D2}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AA7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="17.28515625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" style="8" customWidth="1"/>
-    <col min="4" max="27" width="9.140625" style="8"/>
+    <col min="1" max="2" width="17.33203125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" style="8" customWidth="1"/>
+    <col min="4" max="27" width="9.109375" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>2</v>
       </c>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="C1" s="6"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -3965,7 +3965,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -3973,7 +3973,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -3981,7 +3981,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
@@ -3989,7 +3989,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -3997,7 +3997,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
@@ -4018,16 +4018,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E3F026-F201-4063-9685-60C58AB78B27}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" style="23" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" style="20"/>
+    <col min="1" max="1" width="8.88671875" style="23" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" style="20"/>
     <col min="3" max="5" width="27" style="20" customWidth="1"/>
     <col min="6" max="6" width="27" style="26" customWidth="1"/>
     <col min="7" max="7" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="16" customFormat="1" ht="22.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" s="16" customFormat="1" ht="22.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="27" t="s">
         <v>2</v>
       </c>
@@ -4038,13 +4038,13 @@
         <v>17</v>
       </c>
       <c r="D1" s="28" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E1" s="28" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F1" s="29" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="G1" s="5"/>
       <c r="H1" s="5"/>
@@ -4052,7 +4052,7 @@
       <c r="J1" s="5"/>
       <c r="K1" s="5"/>
     </row>
-    <row r="2" spans="1:11" s="17" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" s="17" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="21" t="s">
         <v>36</v>
       </c>
@@ -4069,10 +4069,10 @@
         <v>36</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
         <v>37</v>
       </c>
@@ -4089,10 +4089,10 @@
         <v>37</v>
       </c>
       <c r="F3" s="25" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
         <v>41</v>
       </c>
@@ -4109,10 +4109,10 @@
         <v>41</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
         <v>42</v>
       </c>
@@ -4129,7 +4129,7 @@
         <v>42</v>
       </c>
       <c r="F5" s="25" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -4157,17 +4157,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63DF2F9F-84FB-4689-BEA6-08562272D65E}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:L13"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" style="14" customWidth="1"/>
-    <col min="2" max="2" width="26.85546875" style="12" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" style="12"/>
+    <col min="2" max="2" width="26.88671875" style="12" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="13"/>
       <c r="B1" s="30" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C1" s="11"/>
       <c r="D1" s="10"/>
@@ -4177,7 +4177,7 @@
       <c r="H1" s="10"/>
       <c r="I1" s="10"/>
     </row>
-    <row r="2" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="31" t="s">
         <v>31</v>
       </c>
@@ -4185,25 +4185,25 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="31"/>
       <c r="B3" s="12" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="31"/>
       <c r="B4" s="12" t="s">
         <v>46</v>
       </c>
       <c r="L4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="31"/>
     </row>
-    <row r="6" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="31" t="s">
         <v>32</v>
       </c>
@@ -4211,25 +4211,25 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="31"/>
       <c r="B7" s="12" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="31"/>
       <c r="B8" s="12" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="31"/>
       <c r="B9" s="12" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" s="31" t="s">
         <v>1</v>
       </c>
@@ -4237,13 +4237,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" s="31"/>
       <c r="B11" s="12" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" s="31" t="s">
         <v>4</v>
       </c>
@@ -4251,7 +4251,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" s="31"/>
       <c r="B13" s="12" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Picked and Dropped Dialogue Working
</commit_message>
<xml_diff>
--- a/Assets/Database/Database.xlsx
+++ b/Assets/Database/Database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tqhie\Unity Projects\Where-To\Assets\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFD0C729-E1C6-4982-B2D5-CB2E69B4F8D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4402BA79-FAE4-4297-BD8A-0CC0A8A476BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0E7384ED-7C35-4E8F-B735-540A4F72621F}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="85">
   <si>
     <t>ID</t>
   </si>
@@ -190,18 +190,6 @@
     <t>PRIORITY</t>
   </si>
   <si>
-    <t>yay/yay1/yay2</t>
-  </si>
-  <si>
-    <t>yo/yo1/yo2</t>
-  </si>
-  <si>
-    <t>yar/yar1/yar2</t>
-  </si>
-  <si>
-    <t>yip/yip1/yip2</t>
-  </si>
-  <si>
     <t xml:space="preserve">GETON </t>
   </si>
   <si>
@@ -260,6 +248,54 @@
   </si>
   <si>
     <t>seven</t>
+  </si>
+  <si>
+    <t>geton_001</t>
+  </si>
+  <si>
+    <t>end_001</t>
+  </si>
+  <si>
+    <t>geton_002</t>
+  </si>
+  <si>
+    <t>geton_003</t>
+  </si>
+  <si>
+    <t>geton_004</t>
+  </si>
+  <si>
+    <t>end_002</t>
+  </si>
+  <si>
+    <t>end_003</t>
+  </si>
+  <si>
+    <t>end_004</t>
+  </si>
+  <si>
+    <t>during_001</t>
+  </si>
+  <si>
+    <t>during_002</t>
+  </si>
+  <si>
+    <t>during_003</t>
+  </si>
+  <si>
+    <t>during_004</t>
+  </si>
+  <si>
+    <t>transition_001</t>
+  </si>
+  <si>
+    <t>transition_002</t>
+  </si>
+  <si>
+    <t>transition_003</t>
+  </si>
+  <si>
+    <t>transition_004</t>
   </si>
 </sst>
 </file>
@@ -1385,7 +1421,7 @@
     <tableColumn id="5" xr3:uid="{94EED148-A6FE-4682-8419-11F273DC0FAC}" name="END" dataDxfId="5"/>
     <tableColumn id="6" xr3:uid="{CF0ECC79-0238-470B-AE20-AE227DD1944E}" name="DURING" dataDxfId="4"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1781,16 +1817,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>22</v>
@@ -1825,16 +1861,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>21</v>
@@ -1846,13 +1882,13 @@
         <v>37</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="R3" s="3"/>
       <c r="S3" s="3"/>
@@ -1869,16 +1905,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>24</v>
@@ -1913,16 +1949,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>25</v>
@@ -1940,7 +1976,7 @@
         <v>10</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -1957,16 +1993,16 @@
         <v>1</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>22</v>
@@ -2001,16 +2037,16 @@
         <v>1</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>26</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>21</v>
@@ -2028,7 +2064,7 @@
         <v>14</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
@@ -2045,16 +2081,16 @@
         <v>1</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>24</v>
@@ -2089,16 +2125,16 @@
         <v>1</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>25</v>
@@ -2116,7 +2152,7 @@
         <v>10</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
@@ -4038,13 +4074,13 @@
         <v>17</v>
       </c>
       <c r="D1" s="28" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E1" s="28" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F1" s="29" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="G1" s="5"/>
       <c r="H1" s="5"/>
@@ -4060,16 +4096,16 @@
         <v>22</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>36</v>
+        <v>81</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>36</v>
+        <v>69</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>49</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -4080,16 +4116,16 @@
         <v>21</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>37</v>
+        <v>74</v>
       </c>
       <c r="F3" s="25" t="s">
-        <v>50</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -4100,16 +4136,16 @@
         <v>24</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>41</v>
+        <v>83</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>41</v>
+        <v>75</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>51</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -4120,23 +4156,24 @@
         <v>25</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>42</v>
+        <v>84</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="F5" s="25" t="s">
-        <v>52</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -4167,7 +4204,7 @@
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="13"/>
       <c r="B1" s="30" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C1" s="11"/>
       <c r="D1" s="10"/>

</xml_diff>